<commit_message>
data: update tax decisions 2026-09-13
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -815,7 +815,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -895,7 +899,7 @@
         <v>46277</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -929,7 +933,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1135,7 +1143,7 @@
         <v>46273</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1261,7 +1269,7 @@
         <v>46273</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -4675,7 +4683,7 @@
         <v>46254</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -4801,7 +4809,7 @@
         <v>46254</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -7497,7 +7505,7 @@
         <v>46246</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -10835,7 +10843,7 @@
         <v>46234</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -10957,7 +10965,7 @@
         <v>46238</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11083,7 +11091,7 @@
         <v>46238</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -11861,7 +11869,7 @@
         <v>46254</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -12377,7 +12385,7 @@
         <v>46229</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -12503,7 +12511,7 @@
         <v>46229</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -17435,7 +17443,7 @@
         <v>46258</v>
       </c>
       <c r="AA135" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB135" s="2" t="inlineStr">
         <is>
@@ -17577,7 +17585,7 @@
         <v>46254</v>
       </c>
       <c r="AA136" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB136" s="2" t="inlineStr">
         <is>
@@ -18519,7 +18527,7 @@
         <v>46258</v>
       </c>
       <c r="AA143" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB143" s="2" t="inlineStr">
         <is>
@@ -22120,7 +22128,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -25208,7 +25216,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25350,7 +25358,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -26174,7 +26182,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -27294,7 +27302,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -27374,7 +27386,7 @@
         <v>46277</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27408,7 +27420,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -27492,7 +27508,7 @@
         <v>46273</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -27618,7 +27634,7 @@
         <v>46273</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -30534,7 +30550,7 @@
         <v>46254</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -30660,7 +30676,7 @@
         <v>46254</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -33098,7 +33114,7 @@
         <v>46246</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -34944,7 +34960,7 @@
         <v>46238</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -35070,7 +35086,7 @@
         <v>46238</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -35426,7 +35442,7 @@
         <v>46254</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -35670,7 +35686,7 @@
         <v>46229</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -35796,7 +35812,7 @@
         <v>46229</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -38968,7 +38984,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -39094,7 +39110,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -40241,7 +40257,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -40367,7 +40383,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -40564,7 +40580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -46826,8 +46842,57 @@
         </is>
       </c>
     </row>
+    <row r="127" ht="54" customHeight="1">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13T17:27:56+08:00</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06 至 2026-09-13</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v>296</v>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G127" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问74页，访问失败215页，持久化待复核208个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M126"/>
+  <autoFilter ref="A1:M127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-14
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$130</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -821,7 +821,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1409,7 +1413,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -27662,7 +27670,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -28014,7 +28022,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -28128,7 +28140,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -41288,7 +41304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M129"/>
+  <dimension ref="A1:M130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -47701,8 +47717,57 @@
         </is>
       </c>
     </row>
+    <row r="130" ht="54" customHeight="1">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14T18:05:09+08:00</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07 至 2026-09-14</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="n">
+        <v>293</v>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G130" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H130" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I130" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问71页，访问失败219页，持久化待复核212个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M129"/>
+  <autoFilter ref="A1:M130"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-15
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46279</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
         <v>46273</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         <v>46273</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -5041,7 +5041,7 @@
         <v>46254</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5167,7 +5167,7 @@
         <v>46254</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -7863,7 +7863,7 @@
         <v>46246</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -11201,7 +11201,7 @@
         <v>46234</v>
       </c>
       <c r="AA86" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB86" s="2" t="inlineStr">
         <is>
@@ -11323,7 +11323,7 @@
         <v>46238</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -11449,7 +11449,7 @@
         <v>46238</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -12227,7 +12227,7 @@
         <v>46254</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12743,7 +12743,7 @@
         <v>46229</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -12869,7 +12869,7 @@
         <v>46229</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -16899,7 +16899,7 @@
         <v>46229</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -17667,7 +17667,7 @@
         <v>46254</v>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
@@ -17801,7 +17801,7 @@
         <v>46258</v>
       </c>
       <c r="AA138" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB138" s="2" t="inlineStr">
         <is>
@@ -17943,7 +17943,7 @@
         <v>46254</v>
       </c>
       <c r="AA139" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB139" s="2" t="inlineStr">
         <is>
@@ -18885,7 +18885,7 @@
         <v>46258</v>
       </c>
       <c r="AA146" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB146" s="2" t="inlineStr">
         <is>
@@ -22490,7 +22490,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -25578,7 +25578,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -25720,7 +25720,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -26544,7 +26544,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -27630,7 +27630,7 @@
         <v>46279</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28228,7 +28228,7 @@
         <v>46273</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -28354,7 +28354,7 @@
         <v>46273</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -31270,7 +31270,7 @@
         <v>46254</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -31396,7 +31396,7 @@
         <v>46254</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -33834,7 +33834,7 @@
         <v>46246</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -35680,7 +35680,7 @@
         <v>46238</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -35806,7 +35806,7 @@
         <v>46238</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -36162,7 +36162,7 @@
         <v>46254</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -36406,7 +36406,7 @@
         <v>46229</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -36532,7 +36532,7 @@
         <v>46229</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -38708,7 +38708,7 @@
         <v>46229</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -39070,7 +39070,7 @@
         <v>46254</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -39708,7 +39708,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -39834,7 +39834,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -39952,7 +39952,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -40981,7 +40981,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -41107,7 +41107,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -41225,7 +41225,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -41304,7 +41304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -47766,8 +47766,57 @@
         </is>
       </c>
     </row>
+    <row r="131" ht="54" customHeight="1">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15T17:22:30+08:00</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08 至 2026-09-15</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="n">
+        <v>292</v>
+      </c>
+      <c r="D131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="G131" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="H131" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I131" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J131" s="2" t="inlineStr"/>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问71页，访问失败218页，持久化待复核211个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M130"/>
+  <autoFilter ref="A1:M131"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-16
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46280</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -815,7 +815,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -895,7 +899,7 @@
         <v>46280</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -929,7 +933,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1009,7 +1017,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1043,7 +1051,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1119,7 +1131,7 @@
         <v>46280</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1153,7 +1165,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1233,7 +1249,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1267,7 +1283,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1347,7 +1367,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1381,7 +1401,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1461,7 +1485,7 @@
         <v>46279</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -5721,7 +5745,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -5847,7 +5871,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -8543,7 +8567,7 @@
         <v>46246</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -11881,7 +11905,7 @@
         <v>46234</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -12003,7 +12027,7 @@
         <v>46238</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -12129,7 +12153,7 @@
         <v>46238</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -12907,7 +12931,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13423,7 +13447,7 @@
         <v>46229</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -13549,7 +13573,7 @@
         <v>46229</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -18481,7 +18505,7 @@
         <v>46258</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -18623,7 +18647,7 @@
         <v>46254</v>
       </c>
       <c r="AA145" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB145" s="2" t="inlineStr">
         <is>
@@ -19565,7 +19589,7 @@
         <v>46258</v>
       </c>
       <c r="AA152" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB152" s="2" t="inlineStr">
         <is>
@@ -23176,7 +23200,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -26264,7 +26288,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -26406,7 +26430,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27230,7 +27254,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28316,7 +28340,7 @@
         <v>46280</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28350,7 +28374,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -28430,7 +28458,7 @@
         <v>46280</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -28464,7 +28492,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -28544,7 +28576,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -28578,7 +28610,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -28654,7 +28690,7 @@
         <v>46280</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -28688,7 +28724,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -28768,7 +28808,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -28802,7 +28842,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -28882,7 +28926,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -28916,7 +28960,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -28996,7 +29044,7 @@
         <v>46279</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -32636,7 +32684,7 @@
         <v>46254</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -32762,7 +32810,7 @@
         <v>46254</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -35200,7 +35248,7 @@
         <v>46246</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -37046,7 +37094,7 @@
         <v>46238</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -37172,7 +37220,7 @@
         <v>46238</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -37528,7 +37576,7 @@
         <v>46254</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -37772,7 +37820,7 @@
         <v>46229</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -37898,7 +37946,7 @@
         <v>46229</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -41080,7 +41128,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -41206,7 +41254,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -42353,7 +42401,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -42479,7 +42527,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -42676,7 +42724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M132"/>
+  <dimension ref="A1:M133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -49240,8 +49288,57 @@
         </is>
       </c>
     </row>
+    <row r="133" ht="54" customHeight="1">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16T17:15:18+08:00</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09 至 2026-09-16</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="n">
+        <v>301</v>
+      </c>
+      <c r="D133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E133" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G133" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H133" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I133" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J133" s="2" t="inlineStr"/>
+      <c r="K133" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问69页，访问失败225页，持久化待复核218个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M132"/>
+  <autoFilter ref="A1:M133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-17
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$136</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1769,7 +1769,7 @@
       </c>
       <c r="AJ10" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -29573,7 +29573,7 @@
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -29699,7 +29699,7 @@
       </c>
       <c r="AJ10" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -43466,7 +43466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M135"/>
+  <dimension ref="A1:M136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50185,8 +50185,57 @@
         </is>
       </c>
     </row>
+    <row r="136" ht="54" customHeight="1">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T17:42:42+08:00</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10 至 2026-09-17</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="n">
+        <v>302</v>
+      </c>
+      <c r="D136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G136" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H136" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I136" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问67页，访问失败230页，持久化待复核223个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M135"/>
+  <autoFilter ref="A1:M136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-18
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$108</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -825,7 +825,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1265,7 +1265,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         <v>46280</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -29011,7 +29011,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -29137,7 +29137,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -29219,7 +29219,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29451,7 +29451,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -29569,7 +29569,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -29683,7 +29683,7 @@
         <v>46280</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -29801,7 +29801,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -29919,7 +29919,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -43978,7 +43978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M137"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50799,8 +50799,57 @@
         </is>
       </c>
     </row>
+    <row r="138" ht="54" customHeight="1">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18T17:16:42+08:00</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11 至 2026-09-18</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="n">
+        <v>316</v>
+      </c>
+      <c r="D138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G138" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H138" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I138" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问74页，访问失败234页，持久化待复核226个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M137"/>
+  <autoFilter ref="A1:M138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-19
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$108</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$139</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46283</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46283</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1265,7 +1265,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         <v>46280</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1615,7 +1615,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1855,7 +1855,7 @@
         <v>46282</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -1981,7 +1981,7 @@
         <v>46282</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         <v>46279</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -6363,7 +6363,7 @@
         <v>46254</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6489,7 +6489,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -9185,7 +9185,7 @@
         <v>46246</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -12523,7 +12523,7 @@
         <v>46234</v>
       </c>
       <c r="AA97" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB97" s="2" t="inlineStr">
         <is>
@@ -12645,7 +12645,7 @@
         <v>46238</v>
       </c>
       <c r="AA98" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB98" s="2" t="inlineStr">
         <is>
@@ -12771,7 +12771,7 @@
         <v>46238</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -13549,7 +13549,7 @@
         <v>46254</v>
       </c>
       <c r="AA105" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB105" s="2" t="inlineStr">
         <is>
@@ -18221,7 +18221,7 @@
         <v>46229</v>
       </c>
       <c r="AA142" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB142" s="2" t="inlineStr">
         <is>
@@ -18989,7 +18989,7 @@
         <v>46254</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -19123,7 +19123,7 @@
         <v>46258</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19265,7 +19265,7 @@
         <v>46254</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -20207,7 +20207,7 @@
         <v>46258</v>
       </c>
       <c r="AA157" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB157" s="2" t="inlineStr">
         <is>
@@ -23827,7 +23827,7 @@
         <v>46234</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -26915,7 +26915,7 @@
         <v>46258</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -27057,7 +27057,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27881,7 +27881,7 @@
         <v>46258</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -28971,7 +28971,7 @@
         <v>46283</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -29097,7 +29097,7 @@
         <v>46283</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -29219,7 +29219,7 @@
         <v>46280</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29451,7 +29451,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -29569,7 +29569,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -29683,7 +29683,7 @@
         <v>46280</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -29801,7 +29801,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -29919,7 +29919,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -30041,7 +30041,7 @@
         <v>46282</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -30167,7 +30167,7 @@
         <v>46282</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -30289,7 +30289,7 @@
         <v>46279</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -33929,7 +33929,7 @@
         <v>46254</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -34055,7 +34055,7 @@
         <v>46254</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -36493,7 +36493,7 @@
         <v>46246</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -38339,7 +38339,7 @@
         <v>46238</v>
       </c>
       <c r="AA79" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB79" s="2" t="inlineStr">
         <is>
@@ -38465,7 +38465,7 @@
         <v>46238</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -38821,7 +38821,7 @@
         <v>46254</v>
       </c>
       <c r="AA83" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB83" s="2" t="inlineStr">
         <is>
@@ -41367,7 +41367,7 @@
         <v>46229</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -41729,7 +41729,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -42382,7 +42382,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -42508,7 +42508,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -42626,7 +42626,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -43655,7 +43655,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -43781,7 +43781,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -43899,7 +43899,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -43978,7 +43978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M138"/>
+  <dimension ref="A1:M139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -50848,8 +50848,57 @@
         </is>
       </c>
     </row>
+    <row r="139" ht="54" customHeight="1">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19T16:45:44+08:00</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12 至 2026-09-19</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="n">
+        <v>316</v>
+      </c>
+      <c r="D139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="G139" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="H139" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I139" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J139" s="2" t="inlineStr"/>
+      <c r="K139" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问67页，访问失败236页，持久化待复核228个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M138"/>
+  <autoFilter ref="A1:M139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-20
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1087,7 +1087,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -21889,7 +21893,11 @@
           <t>附件正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -44742,7 +44750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M141"/>
+  <dimension ref="A1:M142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -51767,8 +51775,57 @@
         </is>
       </c>
     </row>
+    <row r="142" ht="54" customHeight="1">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-20T17:33:46+08:00</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-13 至 2026-09-20</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="D142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G142" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H142" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I142" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问70页，访问失败245页，持久化待复核237个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M141"/>
+  <autoFilter ref="A1:M142"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-21
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$142</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$143</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -785,7 +785,7 @@
         <v>46283</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         <v>46283</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
         <v>46285</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1415,7 +1415,7 @@
         <v>46280</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1647,7 +1647,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1765,7 +1765,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         <v>46280</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -1997,7 +1997,7 @@
         <v>46280</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
         <v>46280</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2237,7 +2237,7 @@
         <v>46282</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
         <v>46282</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2485,7 +2485,7 @@
         <v>46279</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -6745,7 +6745,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -6871,7 +6871,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -9567,7 +9567,7 @@
         <v>46246</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -12905,7 +12905,7 @@
         <v>46234</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -13027,7 +13027,7 @@
         <v>46238</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -13153,7 +13153,7 @@
         <v>46238</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13931,7 +13931,7 @@
         <v>46254</v>
       </c>
       <c r="AA108" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB108" s="2" t="inlineStr">
         <is>
@@ -18603,7 +18603,7 @@
         <v>46229</v>
       </c>
       <c r="AA145" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB145" s="2" t="inlineStr">
         <is>
@@ -19371,7 +19371,7 @@
         <v>46254</v>
       </c>
       <c r="AA151" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB151" s="2" t="inlineStr">
         <is>
@@ -19505,7 +19505,7 @@
         <v>46258</v>
       </c>
       <c r="AA152" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB152" s="2" t="inlineStr">
         <is>
@@ -19647,7 +19647,7 @@
         <v>46254</v>
       </c>
       <c r="AA153" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB153" s="2" t="inlineStr">
         <is>
@@ -20589,7 +20589,7 @@
         <v>46258</v>
       </c>
       <c r="AA160" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
@@ -21855,7 +21855,7 @@
         <v>46285</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24351,7 +24351,7 @@
         <v>46234</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -27439,7 +27439,7 @@
         <v>46258</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -27581,7 +27581,7 @@
         <v>46254</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -28405,7 +28405,7 @@
         <v>46258</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -29497,7 +29497,7 @@
         <v>46283</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -29623,7 +29623,7 @@
         <v>46283</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -29989,7 +29989,7 @@
         <v>46280</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -30221,7 +30221,7 @@
         <v>46280</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -30339,7 +30339,7 @@
         <v>46280</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -30453,7 +30453,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -30571,7 +30571,7 @@
         <v>46280</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -30689,7 +30689,7 @@
         <v>46280</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -30811,7 +30811,7 @@
         <v>46282</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -30937,7 +30937,7 @@
         <v>46282</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -31059,7 +31059,7 @@
         <v>46279</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -34699,7 +34699,7 @@
         <v>46254</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -34825,7 +34825,7 @@
         <v>46254</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -37263,7 +37263,7 @@
         <v>46246</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -39109,7 +39109,7 @@
         <v>46238</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -39235,7 +39235,7 @@
         <v>46238</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -39591,7 +39591,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -42137,7 +42137,7 @@
         <v>46229</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -42499,7 +42499,7 @@
         <v>46254</v>
       </c>
       <c r="AA109" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB109" s="2" t="inlineStr">
         <is>
@@ -43154,7 +43154,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -43280,7 +43280,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -43398,7 +43398,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -44427,7 +44427,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -44553,7 +44553,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -44671,7 +44671,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -44750,7 +44750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M142"/>
+  <dimension ref="A1:M143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -51824,8 +51824,57 @@
         </is>
       </c>
     </row>
+    <row r="143" ht="54" customHeight="1">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-21T17:52:03+08:00</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 至 2026-09-21</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="n">
+        <v>339</v>
+      </c>
+      <c r="D143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G143" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H143" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I143" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问81页，访问失败246页，持久化待复核238个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M142"/>
+  <autoFilter ref="A1:M143"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-22
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$146</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -833,7 +833,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -961,7 +965,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -23955,7 +23963,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -24083,7 +24095,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -48878,7 +48894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M145"/>
+  <dimension ref="A1:M146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -56107,8 +56123,57 @@
         </is>
       </c>
     </row>
+    <row r="146" ht="54" customHeight="1">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T17:35:50+08:00</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15 至 2026-09-22</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="n">
+        <v>334</v>
+      </c>
+      <c r="D146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G146" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H146" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I146" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问76页，访问失败253页，持久化待复核242个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M145"/>
+  <autoFilter ref="A1:M146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-23
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -799,7 +799,7 @@
         <v>46287</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
         <v>46287</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
         <v>46286</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         <v>46286</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1289,7 +1289,7 @@
         <v>46286</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         <v>46286</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         <v>46283</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         <v>46283</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         <v>46285</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         <v>46280</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
         <v>46280</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2781,7 +2781,7 @@
         <v>46280</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2895,7 +2895,7 @@
         <v>46280</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3013,7 +3013,7 @@
         <v>46280</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3131,7 +3131,7 @@
         <v>46280</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8147,7 +8147,7 @@
         <v>46254</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -10843,7 +10843,7 @@
         <v>46246</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -14181,7 +14181,7 @@
         <v>46234</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14303,7 +14303,7 @@
         <v>46238</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14429,7 +14429,7 @@
         <v>46238</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -15207,7 +15207,7 @@
         <v>46254</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -20131,7 +20131,7 @@
         <v>46229</v>
       </c>
       <c r="AA157" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB157" s="2" t="inlineStr">
         <is>
@@ -21159,7 +21159,7 @@
         <v>46254</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -21293,7 +21293,7 @@
         <v>46258</v>
       </c>
       <c r="AA166" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB166" s="2" t="inlineStr">
         <is>
@@ -21435,7 +21435,7 @@
         <v>46254</v>
       </c>
       <c r="AA167" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB167" s="2" t="inlineStr">
         <is>
@@ -22637,7 +22637,7 @@
         <v>46258</v>
       </c>
       <c r="AA176" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB176" s="2" t="inlineStr">
         <is>
@@ -23929,7 +23929,7 @@
         <v>46287</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24061,7 +24061,7 @@
         <v>46287</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -24195,7 +24195,7 @@
         <v>46285</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -26959,7 +26959,7 @@
         <v>46234</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -30047,7 +30047,7 @@
         <v>46258</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -30189,7 +30189,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -31013,7 +31013,7 @@
         <v>46258</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -32105,7 +32105,7 @@
         <v>46286</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32223,7 +32223,7 @@
         <v>46286</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32345,7 +32345,7 @@
         <v>46286</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32467,7 +32467,7 @@
         <v>46286</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32589,7 +32589,7 @@
         <v>46283</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -32715,7 +32715,7 @@
         <v>46283</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -33081,7 +33081,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -33313,7 +33313,7 @@
         <v>46280</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -33431,7 +33431,7 @@
         <v>46280</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -33545,7 +33545,7 @@
         <v>46280</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -33663,7 +33663,7 @@
         <v>46280</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -33781,7 +33781,7 @@
         <v>46280</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -38051,7 +38051,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -38177,7 +38177,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -40615,7 +40615,7 @@
         <v>46246</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -42461,7 +42461,7 @@
         <v>46238</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -42587,7 +42587,7 @@
         <v>46238</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -42943,7 +42943,7 @@
         <v>46254</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -45741,7 +45741,7 @@
         <v>46229</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -46363,7 +46363,7 @@
         <v>46254</v>
       </c>
       <c r="AA119" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB119" s="2" t="inlineStr">
         <is>
@@ -47298,7 +47298,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -47424,7 +47424,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -47542,7 +47542,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -48571,7 +48571,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -48697,7 +48697,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -48815,7 +48815,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46287</v>
+        <v>46288</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -48894,7 +48894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M146"/>
+  <dimension ref="A1:M147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -56172,8 +56172,57 @@
         </is>
       </c>
     </row>
+    <row r="147" ht="54" customHeight="1">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T17:15:54+08:00</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 至 2026-09-23</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="D147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G147" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H147" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I147" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J147" s="2" t="inlineStr"/>
+      <c r="K147" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问79页，访问失败258页，持久化待复核247个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M146"/>
+  <autoFilter ref="A1:M147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-24
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$122</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$149</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -799,7 +799,7 @@
         <v>46287</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
         <v>46287</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
         <v>46286</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         <v>46286</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1289,7 +1289,7 @@
         <v>46286</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1411,7 +1411,7 @@
         <v>46286</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1533,7 +1533,7 @@
         <v>46283</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         <v>46283</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         <v>46285</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         <v>46280</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2663,7 +2663,7 @@
         <v>46280</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2781,7 +2781,7 @@
         <v>46280</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2895,7 +2895,7 @@
         <v>46280</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3013,7 +3013,7 @@
         <v>46280</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3131,7 +3131,7 @@
         <v>46280</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -8021,7 +8021,7 @@
         <v>46254</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8147,7 +8147,7 @@
         <v>46254</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -10843,7 +10843,7 @@
         <v>46246</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -14181,7 +14181,7 @@
         <v>46234</v>
       </c>
       <c r="AA110" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB110" s="2" t="inlineStr">
         <is>
@@ -14303,7 +14303,7 @@
         <v>46238</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -14429,7 +14429,7 @@
         <v>46238</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -15207,7 +15207,7 @@
         <v>46254</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -20131,7 +20131,7 @@
         <v>46229</v>
       </c>
       <c r="AA157" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB157" s="2" t="inlineStr">
         <is>
@@ -21159,7 +21159,7 @@
         <v>46254</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -21293,7 +21293,7 @@
         <v>46258</v>
       </c>
       <c r="AA166" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB166" s="2" t="inlineStr">
         <is>
@@ -21435,7 +21435,7 @@
         <v>46254</v>
       </c>
       <c r="AA167" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB167" s="2" t="inlineStr">
         <is>
@@ -22637,7 +22637,7 @@
         <v>46258</v>
       </c>
       <c r="AA176" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB176" s="2" t="inlineStr">
         <is>
@@ -23929,7 +23929,7 @@
         <v>46287</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24061,7 +24061,7 @@
         <v>46287</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -24195,7 +24195,7 @@
         <v>46285</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -26959,7 +26959,7 @@
         <v>46234</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -30047,7 +30047,7 @@
         <v>46258</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -30189,7 +30189,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -31013,7 +31013,7 @@
         <v>46258</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -32105,7 +32105,7 @@
         <v>46286</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32223,7 +32223,7 @@
         <v>46286</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32345,7 +32345,7 @@
         <v>46286</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -32467,7 +32467,7 @@
         <v>46286</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32589,7 +32589,7 @@
         <v>46283</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -32715,7 +32715,7 @@
         <v>46283</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -33081,7 +33081,7 @@
         <v>46280</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -33313,7 +33313,7 @@
         <v>46280</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -33431,7 +33431,7 @@
         <v>46280</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -33545,7 +33545,7 @@
         <v>46280</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -33663,7 +33663,7 @@
         <v>46280</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -33781,7 +33781,7 @@
         <v>46280</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -38051,7 +38051,7 @@
         <v>46254</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -38177,7 +38177,7 @@
         <v>46254</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -40615,7 +40615,7 @@
         <v>46246</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -42461,7 +42461,7 @@
         <v>46238</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -42587,7 +42587,7 @@
         <v>46238</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -42943,7 +42943,7 @@
         <v>46254</v>
       </c>
       <c r="AA91" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB91" s="2" t="inlineStr">
         <is>
@@ -45741,7 +45741,7 @@
         <v>46229</v>
       </c>
       <c r="AA114" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB114" s="2" t="inlineStr">
         <is>
@@ -46363,7 +46363,7 @@
         <v>46254</v>
       </c>
       <c r="AA119" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB119" s="2" t="inlineStr">
         <is>
@@ -47298,7 +47298,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -47424,7 +47424,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -47542,7 +47542,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -48571,7 +48571,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -48697,7 +48697,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -48815,7 +48815,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46288</v>
+        <v>46289</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -48894,7 +48894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M148"/>
+  <dimension ref="A1:M149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -56270,8 +56270,57 @@
         </is>
       </c>
     </row>
+    <row r="149" ht="54" customHeight="1">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24T17:15:13+08:00</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 至 2026-09-24</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="n">
+        <v>347</v>
+      </c>
+      <c r="D149" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G149" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H149" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I149" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fuji...</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问82页，访问失败260页，持久化待复核249个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M148"/>
+  <autoFilter ref="A1:M149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-25
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -821,7 +821,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -32763,7 +32763,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -32885,7 +32885,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -50130,7 +50130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M151"/>
+  <dimension ref="A1:M152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -57661,8 +57661,57 @@
         </is>
       </c>
     </row>
+    <row r="152" ht="54" customHeight="1">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T17:55:12+08:00</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 至 2026-09-25</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="n">
+        <v>377</v>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G152" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="H152" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I152" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问78页，访问失败278页，持久化待复核267个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M151"/>
+  <autoFilter ref="A1:M152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-26
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$127</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$153</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46290</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46290</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1029,7 +1029,7 @@
         <v>46289</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         <v>46289</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1287,7 +1287,7 @@
         <v>46287</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1419,7 +1419,7 @@
         <v>46287</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         <v>46289</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         <v>46286</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1777,7 +1777,7 @@
         <v>46286</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
         <v>46286</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         <v>46286</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -3041,7 +3041,7 @@
         <v>46280</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
         <v>46280</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3391,7 +3391,7 @@
         <v>46280</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3505,7 +3505,7 @@
         <v>46280</v>
       </c>
       <c r="AA24" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB24" s="2" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
         <v>46280</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3741,7 +3741,7 @@
         <v>46280</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -8757,7 +8757,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -11453,7 +11453,7 @@
         <v>46246</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -14791,7 +14791,7 @@
         <v>46234</v>
       </c>
       <c r="AA115" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB115" s="2" t="inlineStr">
         <is>
@@ -14913,7 +14913,7 @@
         <v>46238</v>
       </c>
       <c r="AA116" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB116" s="2" t="inlineStr">
         <is>
@@ -15039,7 +15039,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -15817,7 +15817,7 @@
         <v>46254</v>
       </c>
       <c r="AA123" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB123" s="2" t="inlineStr">
         <is>
@@ -20741,7 +20741,7 @@
         <v>46229</v>
       </c>
       <c r="AA162" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB162" s="2" t="inlineStr">
         <is>
@@ -21769,7 +21769,7 @@
         <v>46254</v>
       </c>
       <c r="AA170" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB170" s="2" t="inlineStr">
         <is>
@@ -21903,7 +21903,7 @@
         <v>46258</v>
       </c>
       <c r="AA171" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB171" s="2" t="inlineStr">
         <is>
@@ -22045,7 +22045,7 @@
         <v>46254</v>
       </c>
       <c r="AA172" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB172" s="2" t="inlineStr">
         <is>
@@ -23247,7 +23247,7 @@
         <v>46258</v>
       </c>
       <c r="AA181" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB181" s="2" t="inlineStr">
         <is>
@@ -24547,7 +24547,7 @@
         <v>46287</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -24679,7 +24679,7 @@
         <v>46287</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27577,7 +27577,7 @@
         <v>46234</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -30665,7 +30665,7 @@
         <v>46258</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -30807,7 +30807,7 @@
         <v>46254</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -31631,7 +31631,7 @@
         <v>46258</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -32723,7 +32723,7 @@
         <v>46290</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32845,7 +32845,7 @@
         <v>46290</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32971,7 +32971,7 @@
         <v>46289</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -33093,7 +33093,7 @@
         <v>46289</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -33211,7 +33211,7 @@
         <v>46289</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -33333,7 +33333,7 @@
         <v>46286</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -33451,7 +33451,7 @@
         <v>46286</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -33573,7 +33573,7 @@
         <v>46286</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -33695,7 +33695,7 @@
         <v>46286</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -34309,7 +34309,7 @@
         <v>46280</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -34541,7 +34541,7 @@
         <v>46280</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -34659,7 +34659,7 @@
         <v>46280</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -34773,7 +34773,7 @@
         <v>46280</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -34891,7 +34891,7 @@
         <v>46280</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -35009,7 +35009,7 @@
         <v>46280</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -39279,7 +39279,7 @@
         <v>46254</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -39405,7 +39405,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -41843,7 +41843,7 @@
         <v>46246</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -43689,7 +43689,7 @@
         <v>46238</v>
       </c>
       <c r="AA92" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB92" s="2" t="inlineStr">
         <is>
@@ -43815,7 +43815,7 @@
         <v>46238</v>
       </c>
       <c r="AA93" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB93" s="2" t="inlineStr">
         <is>
@@ -44171,7 +44171,7 @@
         <v>46254</v>
       </c>
       <c r="AA96" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB96" s="2" t="inlineStr">
         <is>
@@ -46969,7 +46969,7 @@
         <v>46229</v>
       </c>
       <c r="AA119" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB119" s="2" t="inlineStr">
         <is>
@@ -47591,7 +47591,7 @@
         <v>46254</v>
       </c>
       <c r="AA124" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB124" s="2" t="inlineStr">
         <is>
@@ -48534,7 +48534,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -48660,7 +48660,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -48778,7 +48778,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -49807,7 +49807,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -49933,7 +49933,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -50051,7 +50051,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46290</v>
+        <v>46291</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -50130,7 +50130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M152"/>
+  <dimension ref="A1:M153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -57710,8 +57710,57 @@
         </is>
       </c>
     </row>
+    <row r="153" ht="54" customHeight="1">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26T17:18:42+08:00</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19 至 2026-09-26</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="n">
+        <v>374</v>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G153" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H153" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I153" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M153" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问77页，访问失败281页，持久化待复核270个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M152"/>
+  <autoFilter ref="A1:M153"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-09-30
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$135</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -795,7 +795,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1063,7 +1063,7 @@
         <v>46294</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1189,7 +1189,7 @@
         <v>46294</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         <v>46293</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         <v>46293</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1563,7 +1563,7 @@
         <v>46294</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1597,7 +1597,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1677,7 +1681,7 @@
         <v>46294</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1713,7 +1717,7 @@
       </c>
       <c r="AJ9" s="2" t="inlineStr">
         <is>
-          <t>字段“官方原文链接”存在冲突:保留原值“https://gtm-cn-2r42yzjvn0s.jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”,新值“https://jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”未静默覆盖。</t>
+          <t>字段“官方原文链接”存在冲突:保留原值“https://gtm-cn-2r42yzjvn0s.jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”,新值“https://jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1803,7 @@
         <v>46293</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1925,7 +1929,7 @@
         <v>46293</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2047,7 +2051,7 @@
         <v>46290</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2169,7 +2173,7 @@
         <v>46290</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -3663,7 +3667,7 @@
         <v>46286</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3785,7 +3789,7 @@
         <v>46286</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4805,7 +4809,7 @@
         <v>46280</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5037,7 +5041,7 @@
         <v>46280</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5155,7 +5159,7 @@
         <v>46280</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5269,7 +5273,7 @@
         <v>46280</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5387,7 +5391,7 @@
         <v>46280</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5505,7 +5509,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -10395,7 +10399,7 @@
         <v>46254</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10521,7 +10525,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -13217,7 +13221,7 @@
         <v>46246</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -16555,7 +16559,7 @@
         <v>46234</v>
       </c>
       <c r="AA129" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB129" s="2" t="inlineStr">
         <is>
@@ -16677,7 +16681,7 @@
         <v>46238</v>
       </c>
       <c r="AA130" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB130" s="2" t="inlineStr">
         <is>
@@ -16803,7 +16807,7 @@
         <v>46238</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -17581,7 +17585,7 @@
         <v>46254</v>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
@@ -22505,7 +22509,7 @@
         <v>46229</v>
       </c>
       <c r="AA176" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB176" s="2" t="inlineStr">
         <is>
@@ -23533,7 +23537,7 @@
         <v>46254</v>
       </c>
       <c r="AA184" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB184" s="2" t="inlineStr">
         <is>
@@ -23667,7 +23671,7 @@
         <v>46258</v>
       </c>
       <c r="AA185" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB185" s="2" t="inlineStr">
         <is>
@@ -23809,7 +23813,7 @@
         <v>46254</v>
       </c>
       <c r="AA186" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB186" s="2" t="inlineStr">
         <is>
@@ -25011,7 +25015,7 @@
         <v>46258</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -26330,7 +26334,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -26472,7 +26476,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -26594,7 +26598,7 @@
         <v>46294</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -26628,7 +26632,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -30136,7 +30144,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -33224,7 +33232,7 @@
         <v>46258</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -33366,7 +33374,7 @@
         <v>46254</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -34190,7 +34198,7 @@
         <v>46258</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -35295,7 +35303,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35421,7 +35429,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35547,7 +35555,7 @@
         <v>46293</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35673,7 +35681,7 @@
         <v>46293</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35803,7 @@
         <v>46294</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -35831,7 +35839,7 @@
       </c>
       <c r="AJ6" s="2" t="inlineStr">
         <is>
-          <t>字段“官方原文链接”存在冲突:保留原值“https://gtm-cn-2r42yzjvn0s.jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”,新值“https://jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”未静默覆盖。</t>
+          <t>字段“官方原文链接”存在冲突:保留原值“https://gtm-cn-2r42yzjvn0s.jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”,新值“https://jiangsu.chinatax.gov.cn/art/2026/9/28/art_9193_1788059.html”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -35917,7 +35925,7 @@
         <v>46293</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -36043,7 +36051,7 @@
         <v>46293</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -36165,7 +36173,7 @@
         <v>46290</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -36287,7 +36295,7 @@
         <v>46290</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -37133,7 +37141,7 @@
         <v>46286</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -37255,7 +37263,7 @@
         <v>46286</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -37869,7 +37877,7 @@
         <v>46280</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -38101,7 +38109,7 @@
         <v>46280</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -38219,7 +38227,7 @@
         <v>46280</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -38333,7 +38341,7 @@
         <v>46280</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -38451,7 +38459,7 @@
         <v>46280</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -38569,7 +38577,7 @@
         <v>46280</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -42839,7 +42847,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -42965,7 +42973,7 @@
         <v>46254</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -45403,7 +45411,7 @@
         <v>46246</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -47249,7 +47257,7 @@
         <v>46238</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -47375,7 +47383,7 @@
         <v>46238</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -47731,7 +47739,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -50529,7 +50537,7 @@
         <v>46229</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -51151,7 +51159,7 @@
         <v>46254</v>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB132" s="2" t="inlineStr">
         <is>
@@ -52108,7 +52116,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -52234,7 +52242,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -52352,7 +52360,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -53381,7 +53389,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -53507,7 +53515,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -53625,7 +53633,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -53704,7 +53712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M160"/>
+  <dimension ref="A1:M161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -61700,8 +61708,57 @@
         </is>
       </c>
     </row>
+    <row r="161" ht="54" customHeight="1">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T18:26:29+08:00</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 至 2026-09-30</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="n">
+        <v>416</v>
+      </c>
+      <c r="D161" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G161" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H161" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I161" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问93页，访问失败314页，持久化待复核303个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M160"/>
+  <autoFilter ref="A1:M161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-01
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$135</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -795,7 +795,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1063,7 +1063,7 @@
         <v>46294</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1189,7 +1189,7 @@
         <v>46294</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         <v>46293</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         <v>46293</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
         <v>46294</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46293</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1929,7 +1929,7 @@
         <v>46293</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2051,7 +2051,7 @@
         <v>46290</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
         <v>46290</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -3667,7 +3667,7 @@
         <v>46286</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         <v>46286</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -4809,7 +4809,7 @@
         <v>46280</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -5041,7 +5041,7 @@
         <v>46280</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -5159,7 +5159,7 @@
         <v>46280</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
         <v>46280</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5391,7 +5391,7 @@
         <v>46280</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -5509,7 +5509,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -10399,7 +10399,7 @@
         <v>46254</v>
       </c>
       <c r="AA80" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB80" s="2" t="inlineStr">
         <is>
@@ -10525,7 +10525,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -13221,7 +13221,7 @@
         <v>46246</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -16559,7 +16559,7 @@
         <v>46234</v>
       </c>
       <c r="AA129" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB129" s="2" t="inlineStr">
         <is>
@@ -16681,7 +16681,7 @@
         <v>46238</v>
       </c>
       <c r="AA130" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB130" s="2" t="inlineStr">
         <is>
@@ -16807,7 +16807,7 @@
         <v>46238</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -17585,7 +17585,7 @@
         <v>46254</v>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
@@ -22509,7 +22509,7 @@
         <v>46229</v>
       </c>
       <c r="AA176" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB176" s="2" t="inlineStr">
         <is>
@@ -23537,7 +23537,7 @@
         <v>46254</v>
       </c>
       <c r="AA184" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB184" s="2" t="inlineStr">
         <is>
@@ -23671,7 +23671,7 @@
         <v>46258</v>
       </c>
       <c r="AA185" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB185" s="2" t="inlineStr">
         <is>
@@ -23813,7 +23813,7 @@
         <v>46254</v>
       </c>
       <c r="AA186" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB186" s="2" t="inlineStr">
         <is>
@@ -25015,7 +25015,7 @@
         <v>46258</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -26334,7 +26334,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -26476,7 +26476,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -30144,7 +30144,7 @@
         <v>46234</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -33232,7 +33232,7 @@
         <v>46258</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -33374,7 +33374,7 @@
         <v>46254</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -34198,7 +34198,7 @@
         <v>46258</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -35303,7 +35303,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -35429,7 +35429,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -35555,7 +35555,7 @@
         <v>46293</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -35681,7 +35681,7 @@
         <v>46293</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -35803,7 +35803,7 @@
         <v>46294</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -35925,7 +35925,7 @@
         <v>46293</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -36051,7 +36051,7 @@
         <v>46293</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -36173,7 +36173,7 @@
         <v>46290</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -36295,7 +36295,7 @@
         <v>46290</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -37141,7 +37141,7 @@
         <v>46286</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -37263,7 +37263,7 @@
         <v>46286</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -37877,7 +37877,7 @@
         <v>46280</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -38109,7 +38109,7 @@
         <v>46280</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -38227,7 +38227,7 @@
         <v>46280</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -38341,7 +38341,7 @@
         <v>46280</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -38459,7 +38459,7 @@
         <v>46280</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -38577,7 +38577,7 @@
         <v>46280</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -42847,7 +42847,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -42973,7 +42973,7 @@
         <v>46254</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -45411,7 +45411,7 @@
         <v>46246</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -47257,7 +47257,7 @@
         <v>46238</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -47383,7 +47383,7 @@
         <v>46238</v>
       </c>
       <c r="AA101" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB101" s="2" t="inlineStr">
         <is>
@@ -47739,7 +47739,7 @@
         <v>46254</v>
       </c>
       <c r="AA104" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB104" s="2" t="inlineStr">
         <is>
@@ -50537,7 +50537,7 @@
         <v>46229</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -51159,7 +51159,7 @@
         <v>46254</v>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB132" s="2" t="inlineStr">
         <is>
@@ -52116,7 +52116,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -52242,7 +52242,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -52360,7 +52360,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -53389,7 +53389,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -53515,7 +53515,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -53633,7 +53633,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -53712,7 +53712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M162"/>
+  <dimension ref="A1:M163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -61806,8 +61806,57 @@
         </is>
       </c>
     </row>
+    <row r="163" ht="54" customHeight="1">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01T18:53:34+08:00</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24 至 2026-10-01</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="n">
+        <v>429</v>
+      </c>
+      <c r="D163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E163" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F163" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G163" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="H163" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I163" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fuji...</t>
+        </is>
+      </c>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问88页，访问失败321页，持久化待复核310个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M162"/>
+  <autoFilter ref="A1:M163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-02
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$137</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -795,7 +795,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         <v>46296</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
         <v>46296</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1327,7 @@
         <v>46294</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1453,7 +1453,7 @@
         <v>46294</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1579,7 +1579,7 @@
         <v>46293</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1705,7 +1705,7 @@
         <v>46293</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1945,7 +1945,7 @@
         <v>46294</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2597,7 +2597,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ16" s="2" t="inlineStr"/>
+      <c r="AJ16" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -2715,7 +2719,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ17" s="2" t="inlineStr"/>
+      <c r="AJ17" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -4167,7 +4175,7 @@
         <v>46286</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -4289,7 +4297,7 @@
         <v>46286</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -5309,7 +5317,7 @@
         <v>46280</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5541,7 +5549,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -5659,7 +5667,7 @@
         <v>46280</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -5773,7 +5781,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5899,7 @@
         <v>46280</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6009,7 +6017,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -10899,7 +10907,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -11025,7 +11033,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -13721,7 +13729,7 @@
         <v>46246</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -17059,7 +17067,7 @@
         <v>46234</v>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB133" s="2" t="inlineStr">
         <is>
@@ -17181,7 +17189,7 @@
         <v>46238</v>
       </c>
       <c r="AA134" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB134" s="2" t="inlineStr">
         <is>
@@ -17307,7 +17315,7 @@
         <v>46238</v>
       </c>
       <c r="AA135" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB135" s="2" t="inlineStr">
         <is>
@@ -18085,7 +18093,7 @@
         <v>46254</v>
       </c>
       <c r="AA141" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB141" s="2" t="inlineStr">
         <is>
@@ -23009,7 +23017,7 @@
         <v>46229</v>
       </c>
       <c r="AA180" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB180" s="2" t="inlineStr">
         <is>
@@ -24037,7 +24045,7 @@
         <v>46254</v>
       </c>
       <c r="AA188" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB188" s="2" t="inlineStr">
         <is>
@@ -24171,7 +24179,7 @@
         <v>46258</v>
       </c>
       <c r="AA189" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB189" s="2" t="inlineStr">
         <is>
@@ -24313,7 +24321,7 @@
         <v>46254</v>
       </c>
       <c r="AA190" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB190" s="2" t="inlineStr">
         <is>
@@ -25515,7 +25523,7 @@
         <v>46258</v>
       </c>
       <c r="AA199" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB199" s="2" t="inlineStr">
         <is>
@@ -26840,7 +26848,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -26982,7 +26990,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -27114,7 +27122,7 @@
         <v>46296</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -27154,7 +27162,7 @@
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -27246,7 +27254,7 @@
         <v>46296</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -27286,7 +27294,7 @@
       </c>
       <c r="AJ5" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -30914,7 +30922,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -34002,7 +34010,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -34144,7 +34152,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -34968,7 +34976,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -36077,7 +36085,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -36203,7 +36211,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -36329,7 +36337,7 @@
         <v>46293</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -36455,7 +36463,7 @@
         <v>46293</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -36577,7 +36585,7 @@
         <v>46294</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -37229,7 +37237,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -37347,7 +37359,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -38151,7 +38167,7 @@
         <v>46286</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -38273,7 +38289,7 @@
         <v>46286</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -38887,7 +38903,7 @@
         <v>46280</v>
       </c>
       <c r="AA25" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
@@ -39119,7 +39135,7 @@
         <v>46280</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -39237,7 +39253,7 @@
         <v>46280</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -39351,7 +39367,7 @@
         <v>46280</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -39469,7 +39485,7 @@
         <v>46280</v>
       </c>
       <c r="AA30" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB30" s="2" t="inlineStr">
         <is>
@@ -39587,7 +39603,7 @@
         <v>46280</v>
       </c>
       <c r="AA31" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
@@ -43857,7 +43873,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -43983,7 +43999,7 @@
         <v>46254</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -46421,7 +46437,7 @@
         <v>46246</v>
       </c>
       <c r="AA87" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB87" s="2" t="inlineStr">
         <is>
@@ -48267,7 +48283,7 @@
         <v>46238</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -48393,7 +48409,7 @@
         <v>46238</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -48749,7 +48765,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -51547,7 +51563,7 @@
         <v>46229</v>
       </c>
       <c r="AA129" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB129" s="2" t="inlineStr">
         <is>
@@ -52169,7 +52185,7 @@
         <v>46254</v>
       </c>
       <c r="AA134" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB134" s="2" t="inlineStr">
         <is>
@@ -53134,7 +53150,7 @@
         <v>46296</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -53174,7 +53190,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -53266,7 +53282,7 @@
         <v>46296</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -53306,7 +53322,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>尚未找到官方原文;第三方来源仅作待核验线索。</t>
+          <t>尚未找到官方原文;第三方来源仅作待核验线索。 Excel 与 CSV 历史数据已合并核对。 字段“当事人名称”存在冲突:保留原值“青海天月德物流有限公司湟源分公司”,新值“青海易创科技有限公司”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -53392,7 +53408,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -53518,7 +53534,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -53636,7 +53652,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -54669,7 +54685,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -54795,7 +54811,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -54913,7 +54929,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -54992,7 +55008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M164"/>
+  <dimension ref="A1:M165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -63188,8 +63204,57 @@
         </is>
       </c>
     </row>
+    <row r="165" ht="54" customHeight="1">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T18:27:28+08:00</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 至 2026-10-02</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="D165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E165" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F165" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G165" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H165" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I165" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J165" s="2" t="inlineStr"/>
+      <c r="K165" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问92页，访问失败330页，持久化待复核320个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M164"/>
+  <autoFilter ref="A1:M165"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-03
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -815,7 +815,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -929,7 +933,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1043,7 +1051,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1157,7 +1169,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1271,7 +1287,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1385,7 +1405,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1499,7 +1523,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1613,7 +1641,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1727,7 +1759,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1841,7 +1877,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1955,7 +1995,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2069,7 +2113,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -2183,7 +2231,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -2297,7 +2349,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -2665,7 +2721,7 @@
         <v>46296</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2797,7 +2853,7 @@
         <v>46296</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -28851,7 +28907,7 @@
         <v>46296</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -28983,7 +29039,7 @@
         <v>46296</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -37844,7 +37900,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -37958,7 +38018,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ3" s="2" t="inlineStr"/>
+      <c r="AJ3" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -38072,7 +38136,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ4" s="2" t="inlineStr"/>
+      <c r="AJ4" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -38186,7 +38254,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -38300,7 +38372,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -38414,7 +38490,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -38528,7 +38608,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -38642,7 +38726,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -38756,7 +38844,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -38870,7 +38962,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ11" s="2" t="inlineStr"/>
+      <c r="AJ11" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -38984,7 +39080,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ12" s="2" t="inlineStr"/>
+      <c r="AJ12" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -39098,7 +39198,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ13" s="2" t="inlineStr"/>
+      <c r="AJ13" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -39212,7 +39316,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ14" s="2" t="inlineStr"/>
+      <c r="AJ14" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -39326,7 +39434,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ15" s="2" t="inlineStr"/>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -56608,7 +56720,7 @@
         <v>46296</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -56740,7 +56852,7 @@
         <v>46296</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58466,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M167"/>
+  <dimension ref="A1:M168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -66817,8 +66929,57 @@
         </is>
       </c>
     </row>
+    <row r="168" ht="54" customHeight="1">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T18:24:34+08:00</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-26 至 2026-10-03</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="n">
+        <v>466</v>
+      </c>
+      <c r="D168" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E168" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F168" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G168" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="H168" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I168" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J168" s="2" t="inlineStr"/>
+      <c r="K168" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L168" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fuji...</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问100页，访问失败359页，持久化待复核349个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M167"/>
+  <autoFilter ref="A1:M168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-04
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$169</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -2447,7 +2447,7 @@
         <v>46294</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>46294</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2721,7 +2721,7 @@
         <v>46296</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         <v>46296</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -2979,7 +2979,7 @@
         <v>46294</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3105,7 +3105,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3231,7 +3231,7 @@
         <v>46293</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
         <v>46293</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         <v>46294</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -5945,7 +5945,7 @@
         <v>46286</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         <v>46286</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -7087,7 +7087,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7669,7 +7669,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -12803,7 +12803,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -15499,7 +15499,7 @@
         <v>46246</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -18837,7 +18837,7 @@
         <v>46234</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -18959,7 +18959,7 @@
         <v>46238</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         <v>46238</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -19863,7 +19863,7 @@
         <v>46254</v>
       </c>
       <c r="AA156" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
@@ -24787,7 +24787,7 @@
         <v>46229</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -25815,7 +25815,7 @@
         <v>46254</v>
       </c>
       <c r="AA203" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
@@ -25949,7 +25949,7 @@
         <v>46258</v>
       </c>
       <c r="AA204" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB204" s="2" t="inlineStr">
         <is>
@@ -26091,7 +26091,7 @@
         <v>46254</v>
       </c>
       <c r="AA205" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB205" s="2" t="inlineStr">
         <is>
@@ -27293,7 +27293,7 @@
         <v>46258</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -28633,7 +28633,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28775,7 +28775,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -28907,7 +28907,7 @@
         <v>46296</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46296</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32707,7 +32707,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -35937,7 +35937,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -36761,7 +36761,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -39522,7 +39522,7 @@
         <v>46294</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -39648,7 +39648,7 @@
         <v>46294</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -39774,7 +39774,7 @@
         <v>46293</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -39900,7 +39900,7 @@
         <v>46293</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -40140,7 +40140,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -41722,7 +41722,7 @@
         <v>46286</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -41844,7 +41844,7 @@
         <v>46286</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -42458,7 +42458,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -42690,7 +42690,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -42808,7 +42808,7 @@
         <v>46280</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -42922,7 +42922,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -43040,7 +43040,7 @@
         <v>46280</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -43158,7 +43158,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47428,7 +47428,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -47554,7 +47554,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -49992,7 +49992,7 @@
         <v>46246</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -51838,7 +51838,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -51964,7 +51964,7 @@
         <v>46238</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -52320,7 +52320,7 @@
         <v>46254</v>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB121" s="2" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
         <v>46229</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -55740,7 +55740,7 @@
         <v>46254</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -56720,7 +56720,7 @@
         <v>46296</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -56852,7 +56852,7 @@
         <v>46296</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -56978,7 +56978,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -57104,7 +57104,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -57222,7 +57222,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -58255,7 +58255,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -58381,7 +58381,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58499,7 +58499,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58578,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M168"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -66978,8 +66978,57 @@
         </is>
       </c>
     </row>
+    <row r="169" ht="54" customHeight="1">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04T18:32:20+08:00</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-27 至 2026-10-04</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="n">
+        <v>477</v>
+      </c>
+      <c r="D169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E169" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F169" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="G169" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H169" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I169" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J169" s="2" t="inlineStr"/>
+      <c r="K169" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问97页，访问失败373页，持久化待复核363个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M168"/>
+  <autoFilter ref="A1:M169"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-05
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$171</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1371,7 +1371,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
         <v>46294</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>46294</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2979,7 +2979,7 @@
         <v>46294</v>
       </c>
       <c r="AA20" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB20" s="2" t="inlineStr">
         <is>
@@ -3105,7 +3105,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3231,7 +3231,7 @@
         <v>46293</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -3357,7 +3357,7 @@
         <v>46293</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         <v>46294</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -5945,7 +5945,7 @@
         <v>46286</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         <v>46286</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -7087,7 +7087,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7669,7 +7669,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -12803,7 +12803,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -15499,7 +15499,7 @@
         <v>46246</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -18837,7 +18837,7 @@
         <v>46234</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -18959,7 +18959,7 @@
         <v>46238</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         <v>46238</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -19863,7 +19863,7 @@
         <v>46254</v>
       </c>
       <c r="AA156" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
@@ -24787,7 +24787,7 @@
         <v>46229</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -25815,7 +25815,7 @@
         <v>46254</v>
       </c>
       <c r="AA203" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
@@ -25949,7 +25949,7 @@
         <v>46258</v>
       </c>
       <c r="AA204" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB204" s="2" t="inlineStr">
         <is>
@@ -26091,7 +26091,7 @@
         <v>46254</v>
       </c>
       <c r="AA205" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB205" s="2" t="inlineStr">
         <is>
@@ -27293,7 +27293,7 @@
         <v>46258</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -28633,7 +28633,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28775,7 +28775,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32707,7 +32707,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -35937,7 +35937,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -36761,7 +36761,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -37866,7 +37866,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -37984,7 +37984,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -38102,7 +38102,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -38220,7 +38220,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -38338,7 +38338,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -38456,7 +38456,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -38574,7 +38574,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -38692,7 +38692,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -38810,7 +38810,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -38928,7 +38928,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -39046,7 +39046,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -39164,7 +39164,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -39282,7 +39282,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -39400,7 +39400,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -39522,7 +39522,7 @@
         <v>46294</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -39648,7 +39648,7 @@
         <v>46294</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -39774,7 +39774,7 @@
         <v>46293</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -39900,7 +39900,7 @@
         <v>46293</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -40140,7 +40140,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -41722,7 +41722,7 @@
         <v>46286</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -41844,7 +41844,7 @@
         <v>46286</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -42458,7 +42458,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -42690,7 +42690,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -42808,7 +42808,7 @@
         <v>46280</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -42922,7 +42922,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -43040,7 +43040,7 @@
         <v>46280</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -43158,7 +43158,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47428,7 +47428,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -47554,7 +47554,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -49992,7 +49992,7 @@
         <v>46246</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -51838,7 +51838,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -51964,7 +51964,7 @@
         <v>46238</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -52320,7 +52320,7 @@
         <v>46254</v>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB121" s="2" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
         <v>46229</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -55740,7 +55740,7 @@
         <v>46254</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -56978,7 +56978,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -57104,7 +57104,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -57222,7 +57222,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -58255,7 +58255,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -58381,7 +58381,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58499,7 +58499,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58578,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M170"/>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -67076,8 +67076,57 @@
         </is>
       </c>
     </row>
+    <row r="171" ht="54" customHeight="1">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05T19:23:15+08:00</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 至 2026-10-05</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="D171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F171" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G171" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H171" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I171" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J171" s="2" t="inlineStr"/>
+      <c r="K171" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问88页，访问失败374页，持久化待复核364个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M170"/>
+  <autoFilter ref="A1:M171"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-06
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$173</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1371,7 +1371,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2447,7 +2447,7 @@
         <v>46294</v>
       </c>
       <c r="AA16" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         <v>46294</v>
       </c>
       <c r="AA17" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
@@ -2721,7 +2721,7 @@
         <v>46296</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2853,7 +2853,7 @@
         <v>46296</v>
       </c>
       <c r="AA19" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB19" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         <v>46294</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -5945,7 +5945,7 @@
         <v>46286</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         <v>46286</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -7087,7 +7087,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7669,7 +7669,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -12803,7 +12803,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -15499,7 +15499,7 @@
         <v>46246</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -18837,7 +18837,7 @@
         <v>46234</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -18959,7 +18959,7 @@
         <v>46238</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         <v>46238</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -19863,7 +19863,7 @@
         <v>46254</v>
       </c>
       <c r="AA156" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
@@ -24787,7 +24787,7 @@
         <v>46229</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -25815,7 +25815,7 @@
         <v>46254</v>
       </c>
       <c r="AA203" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
@@ -25949,7 +25949,7 @@
         <v>46258</v>
       </c>
       <c r="AA204" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB204" s="2" t="inlineStr">
         <is>
@@ -26091,7 +26091,7 @@
         <v>46254</v>
       </c>
       <c r="AA205" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB205" s="2" t="inlineStr">
         <is>
@@ -27293,7 +27293,7 @@
         <v>46258</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -28633,7 +28633,7 @@
         <v>46294</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -28775,7 +28775,7 @@
         <v>46294</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -28907,7 +28907,7 @@
         <v>46296</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -29039,7 +29039,7 @@
         <v>46296</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32707,7 +32707,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -35937,7 +35937,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -36761,7 +36761,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -37866,7 +37866,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -37984,7 +37984,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -38102,7 +38102,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -38220,7 +38220,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -38338,7 +38338,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -38456,7 +38456,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -38574,7 +38574,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -38692,7 +38692,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -38810,7 +38810,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -38928,7 +38928,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -39046,7 +39046,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -39164,7 +39164,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -39282,7 +39282,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -39400,7 +39400,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -40140,7 +40140,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -41722,7 +41722,7 @@
         <v>46286</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -41844,7 +41844,7 @@
         <v>46286</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -42458,7 +42458,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -42690,7 +42690,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -42808,7 +42808,7 @@
         <v>46280</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -42922,7 +42922,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -43040,7 +43040,7 @@
         <v>46280</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -43158,7 +43158,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47428,7 +47428,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -47554,7 +47554,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -49992,7 +49992,7 @@
         <v>46246</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -51838,7 +51838,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -51964,7 +51964,7 @@
         <v>46238</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -52320,7 +52320,7 @@
         <v>46254</v>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB121" s="2" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
         <v>46229</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -55740,7 +55740,7 @@
         <v>46254</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -56720,7 +56720,7 @@
         <v>46296</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -56852,7 +56852,7 @@
         <v>46296</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -56978,7 +56978,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -57104,7 +57104,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -57222,7 +57222,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -58255,7 +58255,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -58381,7 +58381,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58499,7 +58499,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58578,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M172"/>
+  <dimension ref="A1:M173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -67174,8 +67174,57 @@
         </is>
       </c>
     </row>
+    <row r="173" ht="54" customHeight="1">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06T19:12:34+08:00</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 至 2026-10-06</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="n">
+        <v>471</v>
+      </c>
+      <c r="D173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E173" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G173" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="H173" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I173" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J173" s="2" t="inlineStr"/>
+      <c r="K173" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M173" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问85页，访问失败377页，持久化待复核367个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M172"/>
+  <autoFilter ref="A1:M173"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-07
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$174</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -899,7 +899,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1371,7 +1371,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1607,7 +1607,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1843,7 +1843,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2079,7 +2079,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2197,7 +2197,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -2315,7 +2315,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -3715,7 +3715,7 @@
         <v>46294</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -5945,7 +5945,7 @@
         <v>46286</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -6067,7 +6067,7 @@
         <v>46286</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -7087,7 +7087,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7437,7 +7437,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7669,7 +7669,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -12803,7 +12803,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -15499,7 +15499,7 @@
         <v>46246</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -18837,7 +18837,7 @@
         <v>46234</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -18959,7 +18959,7 @@
         <v>46238</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         <v>46238</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -19863,7 +19863,7 @@
         <v>46254</v>
       </c>
       <c r="AA156" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
@@ -24787,7 +24787,7 @@
         <v>46229</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -25815,7 +25815,7 @@
         <v>46254</v>
       </c>
       <c r="AA203" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
@@ -25949,7 +25949,7 @@
         <v>46258</v>
       </c>
       <c r="AA204" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB204" s="2" t="inlineStr">
         <is>
@@ -26091,7 +26091,7 @@
         <v>46254</v>
       </c>
       <c r="AA205" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB205" s="2" t="inlineStr">
         <is>
@@ -27293,7 +27293,7 @@
         <v>46258</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -32707,7 +32707,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -35937,7 +35937,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -36761,7 +36761,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -37866,7 +37866,7 @@
         <v>46298</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -37984,7 +37984,7 @@
         <v>46298</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -38102,7 +38102,7 @@
         <v>46298</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -38220,7 +38220,7 @@
         <v>46298</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -38338,7 +38338,7 @@
         <v>46298</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -38456,7 +38456,7 @@
         <v>46298</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -38574,7 +38574,7 @@
         <v>46298</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -38692,7 +38692,7 @@
         <v>46298</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -38810,7 +38810,7 @@
         <v>46298</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -38928,7 +38928,7 @@
         <v>46298</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -39046,7 +39046,7 @@
         <v>46298</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -39164,7 +39164,7 @@
         <v>46298</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -39282,7 +39282,7 @@
         <v>46298</v>
       </c>
       <c r="AA14" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
@@ -39400,7 +39400,7 @@
         <v>46298</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -40140,7 +40140,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -41722,7 +41722,7 @@
         <v>46286</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -41844,7 +41844,7 @@
         <v>46286</v>
       </c>
       <c r="AA35" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB35" s="2" t="inlineStr">
         <is>
@@ -42458,7 +42458,7 @@
         <v>46280</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -42690,7 +42690,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -42808,7 +42808,7 @@
         <v>46280</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -42922,7 +42922,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -43040,7 +43040,7 @@
         <v>46280</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -43158,7 +43158,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47428,7 +47428,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -47554,7 +47554,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -49992,7 +49992,7 @@
         <v>46246</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -51838,7 +51838,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -51964,7 +51964,7 @@
         <v>46238</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -52320,7 +52320,7 @@
         <v>46254</v>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB121" s="2" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
         <v>46229</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -55740,7 +55740,7 @@
         <v>46254</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -56978,7 +56978,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -57104,7 +57104,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -57222,7 +57222,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -58255,7 +58255,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -58381,7 +58381,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58499,7 +58499,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58578,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M174"/>
+  <dimension ref="A1:M175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -67272,8 +67272,57 @@
         </is>
       </c>
     </row>
+    <row r="175" ht="54" customHeight="1">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T19:00:28+08:00</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 至 2026-10-07</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="D175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E175" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G175" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H175" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I175" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J175" s="2" t="inlineStr"/>
+      <c r="K175" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M175" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问80页，访问失败384页，持久化待复核374个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M174"/>
+  <autoFilter ref="A1:M175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-08
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$176</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -3715,7 +3715,7 @@
         <v>46294</v>
       </c>
       <c r="AA26" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         <v>46254</v>
       </c>
       <c r="AA99" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB99" s="2" t="inlineStr">
         <is>
@@ -12803,7 +12803,7 @@
         <v>46254</v>
       </c>
       <c r="AA100" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB100" s="2" t="inlineStr">
         <is>
@@ -15499,7 +15499,7 @@
         <v>46246</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -18837,7 +18837,7 @@
         <v>46234</v>
       </c>
       <c r="AA148" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB148" s="2" t="inlineStr">
         <is>
@@ -18959,7 +18959,7 @@
         <v>46238</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         <v>46238</v>
       </c>
       <c r="AA150" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB150" s="2" t="inlineStr">
         <is>
@@ -19863,7 +19863,7 @@
         <v>46254</v>
       </c>
       <c r="AA156" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB156" s="2" t="inlineStr">
         <is>
@@ -24787,7 +24787,7 @@
         <v>46229</v>
       </c>
       <c r="AA195" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB195" s="2" t="inlineStr">
         <is>
@@ -25815,7 +25815,7 @@
         <v>46254</v>
       </c>
       <c r="AA203" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB203" s="2" t="inlineStr">
         <is>
@@ -25949,7 +25949,7 @@
         <v>46258</v>
       </c>
       <c r="AA204" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB204" s="2" t="inlineStr">
         <is>
@@ -26091,7 +26091,7 @@
         <v>46254</v>
       </c>
       <c r="AA205" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB205" s="2" t="inlineStr">
         <is>
@@ -27293,7 +27293,7 @@
         <v>46258</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -32707,7 +32707,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         <v>46258</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -35937,7 +35937,7 @@
         <v>46254</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -36761,7 +36761,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -40140,7 +40140,7 @@
         <v>46294</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -47428,7 +47428,7 @@
         <v>46254</v>
       </c>
       <c r="AA81" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB81" s="2" t="inlineStr">
         <is>
@@ -47554,7 +47554,7 @@
         <v>46254</v>
       </c>
       <c r="AA82" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB82" s="2" t="inlineStr">
         <is>
@@ -49992,7 +49992,7 @@
         <v>46246</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -51838,7 +51838,7 @@
         <v>46238</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -51964,7 +51964,7 @@
         <v>46238</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -52320,7 +52320,7 @@
         <v>46254</v>
       </c>
       <c r="AA121" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB121" s="2" t="inlineStr">
         <is>
@@ -55118,7 +55118,7 @@
         <v>46229</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -55740,7 +55740,7 @@
         <v>46254</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -56978,7 +56978,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -57104,7 +57104,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -57222,7 +57222,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -58255,7 +58255,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -58381,7 +58381,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -58499,7 +58499,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58578,7 +58578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M176"/>
+  <dimension ref="A1:M177"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -67370,8 +67370,57 @@
         </is>
       </c>
     </row>
+    <row r="177" ht="54" customHeight="1">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T19:18:01+08:00</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01 至 2026-10-08</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="n">
+        <v>463</v>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E177" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="G177" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="H177" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I177" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J177" s="2" t="inlineStr"/>
+      <c r="K177" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M177" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问75页，访问失败387页，持久化待复核377个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M176"/>
+  <autoFilter ref="A1:M177"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-10
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$182</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -815,7 +815,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -895,7 +899,7 @@
         <v>46304</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -39092,7 +39096,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ2" s="2" t="inlineStr"/>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -39172,7 +39180,7 @@
         <v>46304</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -60374,7 +60382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M181"/>
+  <dimension ref="A1:M182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -69423,8 +69431,57 @@
         </is>
       </c>
     </row>
+    <row r="182" ht="54" customHeight="1">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T19:01:08+08:00</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03 至 2026-10-10</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="D182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E182" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G182" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H182" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I182" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J182" s="2" t="inlineStr"/>
+      <c r="K182" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问82页，访问失败392页，持久化待复核382个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M181"/>
+  <autoFilter ref="A1:M182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-11
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$157</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$183</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46305</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         <v>46294</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -4569,7 +4569,7 @@
         <v>46296</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -4691,7 +4691,7 @@
         <v>46296</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -6181,7 +6181,7 @@
         <v>46286</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -6303,7 +6303,7 @@
         <v>46286</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -7555,7 +7555,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -7787,7 +7787,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -7905,7 +7905,7 @@
         <v>46280</v>
       </c>
       <c r="AA60" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB60" s="2" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
         <v>46280</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -13035,7 +13035,7 @@
         <v>46254</v>
       </c>
       <c r="AA102" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB102" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         <v>46254</v>
       </c>
       <c r="AA103" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB103" s="2" t="inlineStr">
         <is>
@@ -16101,7 +16101,7 @@
         <v>46246</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -19439,7 +19439,7 @@
         <v>46234</v>
       </c>
       <c r="AA153" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB153" s="2" t="inlineStr">
         <is>
@@ -19561,7 +19561,7 @@
         <v>46238</v>
       </c>
       <c r="AA154" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB154" s="2" t="inlineStr">
         <is>
@@ -19687,7 +19687,7 @@
         <v>46238</v>
       </c>
       <c r="AA155" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB155" s="2" t="inlineStr">
         <is>
@@ -20465,7 +20465,7 @@
         <v>46254</v>
       </c>
       <c r="AA161" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB161" s="2" t="inlineStr">
         <is>
@@ -25679,7 +25679,7 @@
         <v>46229</v>
       </c>
       <c r="AA202" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB202" s="2" t="inlineStr">
         <is>
@@ -26707,7 +26707,7 @@
         <v>46254</v>
       </c>
       <c r="AA210" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB210" s="2" t="inlineStr">
         <is>
@@ -26841,7 +26841,7 @@
         <v>46258</v>
       </c>
       <c r="AA211" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB211" s="2" t="inlineStr">
         <is>
@@ -26983,7 +26983,7 @@
         <v>46254</v>
       </c>
       <c r="AA212" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB212" s="2" t="inlineStr">
         <is>
@@ -28185,7 +28185,7 @@
         <v>46258</v>
       </c>
       <c r="AA221" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB221" s="2" t="inlineStr">
         <is>
@@ -33609,7 +33609,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -36987,7 +36987,7 @@
         <v>46258</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -37129,7 +37129,7 @@
         <v>46254</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -37953,7 +37953,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -39062,7 +39062,7 @@
         <v>46305</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -41572,7 +41572,7 @@
         <v>46294</v>
       </c>
       <c r="AA23" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
@@ -42190,7 +42190,7 @@
         <v>46296</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -42312,7 +42312,7 @@
         <v>46296</v>
       </c>
       <c r="AA29" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
@@ -43154,7 +43154,7 @@
         <v>46286</v>
       </c>
       <c r="AA36" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
@@ -43276,7 +43276,7 @@
         <v>46286</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -43890,7 +43890,7 @@
         <v>46280</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -44122,7 +44122,7 @@
         <v>46280</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -44240,7 +44240,7 @@
         <v>46280</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -44354,7 +44354,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -44472,7 +44472,7 @@
         <v>46280</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -44590,7 +44590,7 @@
         <v>46280</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -48982,7 +48982,7 @@
         <v>46254</v>
       </c>
       <c r="AA84" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB84" s="2" t="inlineStr">
         <is>
@@ -49108,7 +49108,7 @@
         <v>46254</v>
       </c>
       <c r="AA85" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB85" s="2" t="inlineStr">
         <is>
@@ -51790,7 +51790,7 @@
         <v>46246</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -53636,7 +53636,7 @@
         <v>46238</v>
       </c>
       <c r="AA122" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB122" s="2" t="inlineStr">
         <is>
@@ -53762,7 +53762,7 @@
         <v>46238</v>
       </c>
       <c r="AA123" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB123" s="2" t="inlineStr">
         <is>
@@ -54118,7 +54118,7 @@
         <v>46254</v>
       </c>
       <c r="AA126" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB126" s="2" t="inlineStr">
         <is>
@@ -56916,7 +56916,7 @@
         <v>46229</v>
       </c>
       <c r="AA149" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB149" s="2" t="inlineStr">
         <is>
@@ -57538,7 +57538,7 @@
         <v>46254</v>
       </c>
       <c r="AA154" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB154" s="2" t="inlineStr">
         <is>
@@ -58782,7 +58782,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -58908,7 +58908,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -59026,7 +59026,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -60059,7 +60059,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -60185,7 +60185,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -60303,7 +60303,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -60382,7 +60382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M182"/>
+  <dimension ref="A1:M183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -69480,8 +69480,57 @@
         </is>
       </c>
     </row>
+    <row r="183" ht="54" customHeight="1">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11T18:46:11+08:00</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-04 至 2026-10-11</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="D183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E183" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="G183" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H183" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I183" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fuji...</t>
+        </is>
+      </c>
+      <c r="M183" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问88页，访问失败393页，持久化待复核383个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M182"/>
+  <autoFilter ref="A1:M183"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-12
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$161</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$184</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -943,7 +943,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
         <v>46306</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1307,7 +1307,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1391,7 +1395,7 @@
         <v>46306</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1425,7 +1429,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -4439,7 +4447,7 @@
         <v>46294</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -5057,7 +5065,7 @@
         <v>46296</v>
       </c>
       <c r="AA37" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
@@ -5179,7 +5187,7 @@
         <v>46296</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -6669,7 +6677,7 @@
         <v>46286</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6791,7 +6799,7 @@
         <v>46286</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -7811,7 +7819,7 @@
         <v>46280</v>
       </c>
       <c r="AA59" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB59" s="2" t="inlineStr">
         <is>
@@ -8043,7 +8051,7 @@
         <v>46280</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8161,7 +8169,7 @@
         <v>46280</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -8275,7 +8283,7 @@
         <v>46280</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8393,7 +8401,7 @@
         <v>46280</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -8511,7 +8519,7 @@
         <v>46280</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -13523,7 +13531,7 @@
         <v>46254</v>
       </c>
       <c r="AA106" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB106" s="2" t="inlineStr">
         <is>
@@ -13649,7 +13657,7 @@
         <v>46254</v>
       </c>
       <c r="AA107" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB107" s="2" t="inlineStr">
         <is>
@@ -16589,7 +16597,7 @@
         <v>46246</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -19927,7 +19935,7 @@
         <v>46234</v>
       </c>
       <c r="AA157" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB157" s="2" t="inlineStr">
         <is>
@@ -20049,7 +20057,7 @@
         <v>46238</v>
       </c>
       <c r="AA158" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB158" s="2" t="inlineStr">
         <is>
@@ -20175,7 +20183,7 @@
         <v>46238</v>
       </c>
       <c r="AA159" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB159" s="2" t="inlineStr">
         <is>
@@ -26167,7 +26175,7 @@
         <v>46229</v>
       </c>
       <c r="AA206" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB206" s="2" t="inlineStr">
         <is>
@@ -27195,7 +27203,7 @@
         <v>46254</v>
       </c>
       <c r="AA214" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB214" s="2" t="inlineStr">
         <is>
@@ -28673,7 +28681,7 @@
         <v>46258</v>
       </c>
       <c r="AA225" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB225" s="2" t="inlineStr">
         <is>
@@ -34103,7 +34111,7 @@
         <v>46234</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -38447,7 +38455,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -39718,7 +39726,7 @@
       </c>
       <c r="AJ3" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -39844,7 +39852,7 @@
       </c>
       <c r="AJ4" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -40048,7 +40056,7 @@
         <v>46306</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -40082,7 +40090,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -40166,7 +40178,7 @@
         <v>46306</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -40200,7 +40212,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -42554,7 +42570,7 @@
         <v>46294</v>
       </c>
       <c r="AA27" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB27" s="2" t="inlineStr">
         <is>
@@ -43172,7 +43188,7 @@
         <v>46296</v>
       </c>
       <c r="AA32" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB32" s="2" t="inlineStr">
         <is>
@@ -43294,7 +43310,7 @@
         <v>46296</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -44136,7 +44152,7 @@
         <v>46286</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -44258,7 +44274,7 @@
         <v>46286</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -44872,7 +44888,7 @@
         <v>46280</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -45104,7 +45120,7 @@
         <v>46280</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -45222,7 +45238,7 @@
         <v>46280</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -45336,7 +45352,7 @@
         <v>46280</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -45454,7 +45470,7 @@
         <v>46280</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -45572,7 +45588,7 @@
         <v>46280</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -49964,7 +49980,7 @@
         <v>46254</v>
       </c>
       <c r="AA88" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB88" s="2" t="inlineStr">
         <is>
@@ -50090,7 +50106,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -52772,7 +52788,7 @@
         <v>46246</v>
       </c>
       <c r="AA111" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB111" s="2" t="inlineStr">
         <is>
@@ -54618,7 +54634,7 @@
         <v>46238</v>
       </c>
       <c r="AA126" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB126" s="2" t="inlineStr">
         <is>
@@ -54744,7 +54760,7 @@
         <v>46238</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -57898,7 +57914,7 @@
         <v>46229</v>
       </c>
       <c r="AA153" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB153" s="2" t="inlineStr">
         <is>
@@ -58520,7 +58536,7 @@
         <v>46254</v>
       </c>
       <c r="AA158" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB158" s="2" t="inlineStr">
         <is>
@@ -59770,7 +59786,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -59896,7 +59912,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -60014,7 +60030,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -61047,7 +61063,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -61173,7 +61189,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -61291,7 +61307,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -61370,7 +61386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M184"/>
+  <dimension ref="A1:M185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -70570,8 +70586,57 @@
         </is>
       </c>
     </row>
+    <row r="185" ht="54" customHeight="1">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12T19:52:13+08:00</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-05 至 2026-10-12</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="n">
+        <v>496</v>
+      </c>
+      <c r="D185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E185" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="G185" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H185" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I185" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
+      <c r="K185" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L185" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问74页，访问失败407页，持久化待复核397个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M184"/>
+  <autoFilter ref="A1:M185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-14
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$189</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -797,7 +797,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>46308</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1586,7 +1586,7 @@
         <v>46306</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
         <v>46306</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         <v>46304</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
         <v>46306</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2078,7 +2078,7 @@
         <v>46306</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         <v>46308</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="AJ13" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“苏州税稽处〔2026〕164号”,新值“苏州税稽处〔2026〕162号”未静默覆盖。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“苏州税稽处〔2026〕164号”,新值“苏州税稽处〔2026〕162号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -5248,7 +5248,7 @@
         <v>46294</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>46296</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         <v>46296</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -7478,7 +7478,7 @@
         <v>46286</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7600,7 +7600,7 @@
         <v>46286</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -8620,7 +8620,7 @@
         <v>46280</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8852,7 +8852,7 @@
         <v>46280</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -8970,7 +8970,7 @@
         <v>46280</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9084,7 +9084,7 @@
         <v>46280</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9202,7 +9202,7 @@
         <v>46280</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9320,7 +9320,7 @@
         <v>46280</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -14332,7 +14332,7 @@
         <v>46254</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14458,7 +14458,7 @@
         <v>46254</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -17398,7 +17398,7 @@
         <v>46246</v>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
@@ -20736,7 +20736,7 @@
         <v>46234</v>
       </c>
       <c r="AA163" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB163" s="2" t="inlineStr">
         <is>
@@ -20858,7 +20858,7 @@
         <v>46238</v>
       </c>
       <c r="AA164" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB164" s="2" t="inlineStr">
         <is>
@@ -20984,7 +20984,7 @@
         <v>46238</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -21762,7 +21762,7 @@
         <v>46254</v>
       </c>
       <c r="AA171" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB171" s="2" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         <v>46258</v>
       </c>
       <c r="AA222" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB222" s="2" t="inlineStr">
         <is>
@@ -28402,7 +28402,7 @@
         <v>46254</v>
       </c>
       <c r="AA223" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB223" s="2" t="inlineStr">
         <is>
@@ -29604,7 +29604,7 @@
         <v>46258</v>
       </c>
       <c r="AA232" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB232" s="2" t="inlineStr">
         <is>
@@ -30975,7 +30975,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -31117,7 +31117,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31243,7 +31243,7 @@
         <v>46308</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31380,7 +31380,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31519,7 +31519,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -35730,7 +35730,7 @@
         <v>46234</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -39108,7 +39108,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -39250,7 +39250,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -40074,7 +40074,7 @@
         <v>46258</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -41315,7 +41315,7 @@
         <v>46306</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -41441,7 +41441,7 @@
         <v>46306</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -41563,7 +41563,7 @@
         <v>46304</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -41685,7 +41685,7 @@
         <v>46306</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -41807,7 +41807,7 @@
         <v>46306</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -41925,7 +41925,7 @@
         <v>46308</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -41961,7 +41961,7 @@
       </c>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
-          <t>字段“决定书文号”存在冲突:保留原值“苏州税稽处〔2026〕164号”,新值“苏州税稽处〔2026〕162号”未静默覆盖。</t>
+          <t>字段“决定书文号”存在冲突:保留原值“苏州税稽处〔2026〕164号”,新值“苏州税稽处〔2026〕162号”未静默覆盖。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -44317,7 +44317,7 @@
         <v>46294</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -44935,7 +44935,7 @@
         <v>46296</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -45057,7 +45057,7 @@
         <v>46296</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -45899,7 +45899,7 @@
         <v>46286</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -46021,7 +46021,7 @@
         <v>46286</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -46635,7 +46635,7 @@
         <v>46280</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -46867,7 +46867,7 @@
         <v>46280</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -46985,7 +46985,7 @@
         <v>46280</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -47099,7 +47099,7 @@
         <v>46280</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -47217,7 +47217,7 @@
         <v>46280</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -47335,7 +47335,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -51727,7 +51727,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -51853,7 +51853,7 @@
         <v>46254</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -54535,7 +54535,7 @@
         <v>46246</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -56381,7 +56381,7 @@
         <v>46238</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -56507,7 +56507,7 @@
         <v>46238</v>
       </c>
       <c r="AA128" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB128" s="2" t="inlineStr">
         <is>
@@ -56863,7 +56863,7 @@
         <v>46254</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -61658,7 +61658,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -61784,7 +61784,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -62935,7 +62935,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -63061,7 +63061,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -63258,7 +63258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M188"/>
+  <dimension ref="A1:M189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -72666,8 +72666,57 @@
         </is>
       </c>
     </row>
+    <row r="189" ht="54" customHeight="1">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:27:56+08:00</t>
+        </is>
+      </c>
+      <c r="B189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 至 2026-10-14</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="n">
+        <v>525</v>
+      </c>
+      <c r="D189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E189" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F189" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G189" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H189" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I189" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J189" s="2" t="inlineStr"/>
+      <c r="K189" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/qzsswj/xxgk/sjxxgk/qtgg_23603/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /qzsswj/xxgk/sjxxgk/qtgg_23603/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinata...</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问79页，访问失败418页，持久化待复核409个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M188"/>
+  <autoFilter ref="A1:M189"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-15
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$190</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$191</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -797,7 +797,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -939,7 +939,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>46308</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1202,7 +1202,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1586,7 +1586,7 @@
         <v>46306</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1712,7 +1712,7 @@
         <v>46306</v>
       </c>
       <c r="AA9" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB9" s="2" t="inlineStr">
         <is>
@@ -1834,7 +1834,7 @@
         <v>46304</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
         <v>46306</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2078,7 +2078,7 @@
         <v>46306</v>
       </c>
       <c r="AA12" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
@@ -2196,7 +2196,7 @@
         <v>46308</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
         <v>46294</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -5866,7 +5866,7 @@
         <v>46296</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -5988,7 +5988,7 @@
         <v>46296</v>
       </c>
       <c r="AA44" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
@@ -7478,7 +7478,7 @@
         <v>46286</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -7600,7 +7600,7 @@
         <v>46286</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -8620,7 +8620,7 @@
         <v>46280</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -8852,7 +8852,7 @@
         <v>46280</v>
       </c>
       <c r="AA67" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB67" s="2" t="inlineStr">
         <is>
@@ -8970,7 +8970,7 @@
         <v>46280</v>
       </c>
       <c r="AA68" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB68" s="2" t="inlineStr">
         <is>
@@ -9084,7 +9084,7 @@
         <v>46280</v>
       </c>
       <c r="AA69" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB69" s="2" t="inlineStr">
         <is>
@@ -9202,7 +9202,7 @@
         <v>46280</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9320,7 +9320,7 @@
         <v>46280</v>
       </c>
       <c r="AA71" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB71" s="2" t="inlineStr">
         <is>
@@ -14332,7 +14332,7 @@
         <v>46254</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -14458,7 +14458,7 @@
         <v>46254</v>
       </c>
       <c r="AA113" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB113" s="2" t="inlineStr">
         <is>
@@ -17398,7 +17398,7 @@
         <v>46246</v>
       </c>
       <c r="AA137" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB137" s="2" t="inlineStr">
         <is>
@@ -20736,7 +20736,7 @@
         <v>46234</v>
       </c>
       <c r="AA163" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB163" s="2" t="inlineStr">
         <is>
@@ -20858,7 +20858,7 @@
         <v>46238</v>
       </c>
       <c r="AA164" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB164" s="2" t="inlineStr">
         <is>
@@ -20984,7 +20984,7 @@
         <v>46238</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -21762,7 +21762,7 @@
         <v>46254</v>
       </c>
       <c r="AA171" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB171" s="2" t="inlineStr">
         <is>
@@ -27098,7 +27098,7 @@
         <v>46229</v>
       </c>
       <c r="AA213" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB213" s="2" t="inlineStr">
         <is>
@@ -28126,7 +28126,7 @@
         <v>46254</v>
       </c>
       <c r="AA221" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB221" s="2" t="inlineStr">
         <is>
@@ -28260,7 +28260,7 @@
         <v>46258</v>
       </c>
       <c r="AA222" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB222" s="2" t="inlineStr">
         <is>
@@ -28402,7 +28402,7 @@
         <v>46254</v>
       </c>
       <c r="AA223" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB223" s="2" t="inlineStr">
         <is>
@@ -29604,7 +29604,7 @@
         <v>46258</v>
       </c>
       <c r="AA232" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB232" s="2" t="inlineStr">
         <is>
@@ -30975,7 +30975,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -31117,7 +31117,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31243,7 +31243,7 @@
         <v>46308</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -31380,7 +31380,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -31519,7 +31519,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -35730,7 +35730,7 @@
         <v>46234</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -39108,7 +39108,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -39250,7 +39250,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -40074,7 +40074,7 @@
         <v>46258</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -41315,7 +41315,7 @@
         <v>46306</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -41441,7 +41441,7 @@
         <v>46306</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -41563,7 +41563,7 @@
         <v>46304</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -41685,7 +41685,7 @@
         <v>46306</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -41807,7 +41807,7 @@
         <v>46306</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -41925,7 +41925,7 @@
         <v>46308</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -44317,7 +44317,7 @@
         <v>46294</v>
       </c>
       <c r="AA28" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
@@ -44935,7 +44935,7 @@
         <v>46296</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -45057,7 +45057,7 @@
         <v>46296</v>
       </c>
       <c r="AA34" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB34" s="2" t="inlineStr">
         <is>
@@ -45899,7 +45899,7 @@
         <v>46286</v>
       </c>
       <c r="AA41" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB41" s="2" t="inlineStr">
         <is>
@@ -46021,7 +46021,7 @@
         <v>46286</v>
       </c>
       <c r="AA42" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
@@ -46635,7 +46635,7 @@
         <v>46280</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -46867,7 +46867,7 @@
         <v>46280</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -46985,7 +46985,7 @@
         <v>46280</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -47099,7 +47099,7 @@
         <v>46280</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -47217,7 +47217,7 @@
         <v>46280</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -47335,7 +47335,7 @@
         <v>46280</v>
       </c>
       <c r="AA53" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
@@ -51727,7 +51727,7 @@
         <v>46254</v>
       </c>
       <c r="AA89" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB89" s="2" t="inlineStr">
         <is>
@@ -51853,7 +51853,7 @@
         <v>46254</v>
       </c>
       <c r="AA90" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB90" s="2" t="inlineStr">
         <is>
@@ -54535,7 +54535,7 @@
         <v>46246</v>
       </c>
       <c r="AA112" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB112" s="2" t="inlineStr">
         <is>
@@ -56381,7 +56381,7 @@
         <v>46238</v>
       </c>
       <c r="AA127" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB127" s="2" t="inlineStr">
         <is>
@@ -56507,7 +56507,7 @@
         <v>46238</v>
       </c>
       <c r="AA128" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB128" s="2" t="inlineStr">
         <is>
@@ -56863,7 +56863,7 @@
         <v>46254</v>
       </c>
       <c r="AA131" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB131" s="2" t="inlineStr">
         <is>
@@ -59783,7 +59783,7 @@
         <v>46229</v>
       </c>
       <c r="AA155" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB155" s="2" t="inlineStr">
         <is>
@@ -60405,7 +60405,7 @@
         <v>46254</v>
       </c>
       <c r="AA160" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
@@ -61658,7 +61658,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -61784,7 +61784,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -61902,7 +61902,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -62935,7 +62935,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -63061,7 +63061,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -63179,7 +63179,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -63258,7 +63258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M190"/>
+  <dimension ref="A1:M191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -72764,8 +72764,57 @@
         </is>
       </c>
     </row>
+    <row r="191" ht="54" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15T17:05:57+08:00</t>
+        </is>
+      </c>
+      <c r="B191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 至 2026-10-15</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="n">
+        <v>531</v>
+      </c>
+      <c r="D191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E191" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G191" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H191" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I191" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J191" s="2" t="inlineStr"/>
+      <c r="K191" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /fzsswj/xxgk/gsgg/qtl/ (Caused by NewConnectionError("HTTPSConnection(host='fujian.chinatax.gov.cn', port=44...</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问82页，访问失败430页，持久化待复核421个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M190"/>
+  <autoFilter ref="A1:M191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-17
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$168</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46311</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -821,7 +821,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
         <v>46311</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         <v>46311</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         <v>46311</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1185,7 +1185,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1269,7 +1273,7 @@
         <v>46311</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1303,7 +1307,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1399,7 +1407,7 @@
         <v>46308</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1541,7 +1549,7 @@
         <v>46308</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1776,7 +1784,7 @@
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>我局于2025年6月16日起,对你2020年1月1日-2020年12月31日期间的涉税情况进行检查,确认你有如下违法事实,并作出如下处罚决定: 根据《税务处理决定书》(鄂税三稽处〔2026〕8号)认定你存在以下违法事实: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 根据《中华人民共和国税收征收管理法》(2015年4月24日发布的主席令第二十三号修订)第六十四条第二款:“纳税人不进行纳税申报,不缴或者少缴应纳税款的,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 根据《内蒙古自治区国家税务局内蒙古自治区地方税务局关于发布〈内蒙古自治区税务行政处罚裁量基准〉的公告》(内蒙古自治区国家税务局内蒙古自治区地方税务局公告2017年第8号):“三、违反纳税申报管理类(三)纳税人不进行纳税申报,不缴或者少缴应纳税款的。 《中华人民共和国税收征收管理法》第六十四条第二款,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 1.不缴或者少缴税款100万元以下的,处百分之五十以上一倍以下罚款; ”之规定,决定对你个人不进行纳税申报造成少缴税款2,129.45元处以0.5倍罚款,即1,064.73元。</t>
+          <t>我局于2025年6月16日起,对你(地址:内蒙古鄂尔多斯市伊金霍洛旗纳林陶亥镇道劳岱村沟门社034号)2020年1月1日-2020年12月31日期间的涉税情况进行检查,违法事实及处理决定如下: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 ”之规定,对你少缴的个人所得税税款,按日加收滞纳税款万分之五的滞纳金。</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
@@ -1784,13 +1792,15 @@
           <t>个人所得税</t>
         </is>
       </c>
-      <c r="R10" s="3" t="n"/>
+      <c r="R10" s="3" t="n">
+        <v>2129.45</v>
+      </c>
       <c r="S10" s="3" t="n"/>
       <c r="T10" s="3" t="n"/>
       <c r="U10" s="3" t="n"/>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>综上所述,对你共处罚款1,064.73元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+          <t>你在2020年应税收入为163,804.00元,应纳税额=163,804.00*1.3%=2,129.45元,应补缴个人所得税2,129.45元。 综上,你在2020年应税收入为163,804.00元,应补缴个人所得税2,129.45元,并就上述税款按日加收万分之五的滞纳金。</t>
         </is>
       </c>
       <c r="W10" s="4" t="n">
@@ -1804,7 +1814,7 @@
         <v>46308</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1847,7 +1857,7 @@
         <is>
           <t>Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/t20261013_898073.html”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202610/t20261013_898073.html”未静默覆盖。 字段“附件链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013417006903908.docx”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202610/P020261013417006903908.docx”未静默覆盖。 字段“页面标题”存在冲突:保留原值“国家税务总局内蒙古自治区税务局-
 旗县局通知公告”,新值“国家税务总局内蒙古自治区税务局-
-通知公告”未静默覆盖。</t>
+通知公告”未静默覆盖。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。 字段“附件链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013417006903908.docx”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013557090721134.docx”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1955,7 @@
         <v>46308</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2440,7 +2450,7 @@
         <v>46304</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2802,7 +2812,7 @@
         <v>46308</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -5854,7 +5864,7 @@
         <v>46294</v>
       </c>
       <c r="AA43" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB43" s="2" t="inlineStr">
         <is>
@@ -6472,7 +6482,7 @@
         <v>46296</v>
       </c>
       <c r="AA48" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
@@ -6594,7 +6604,7 @@
         <v>46296</v>
       </c>
       <c r="AA49" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
@@ -8084,7 +8094,7 @@
         <v>46286</v>
       </c>
       <c r="AA61" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
@@ -8206,7 +8216,7 @@
         <v>46286</v>
       </c>
       <c r="AA62" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
@@ -9226,7 +9236,7 @@
         <v>46280</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -9458,7 +9468,7 @@
         <v>46280</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9576,7 +9586,7 @@
         <v>46280</v>
       </c>
       <c r="AA73" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB73" s="2" t="inlineStr">
         <is>
@@ -9690,7 +9700,7 @@
         <v>46280</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -9808,7 +9818,7 @@
         <v>46280</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -9926,7 +9936,7 @@
         <v>46280</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -14938,7 +14948,7 @@
         <v>46254</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -15064,7 +15074,7 @@
         <v>46254</v>
       </c>
       <c r="AA118" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB118" s="2" t="inlineStr">
         <is>
@@ -18004,7 +18014,7 @@
         <v>46246</v>
       </c>
       <c r="AA142" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB142" s="2" t="inlineStr">
         <is>
@@ -21342,7 +21352,7 @@
         <v>46234</v>
       </c>
       <c r="AA168" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB168" s="2" t="inlineStr">
         <is>
@@ -21464,7 +21474,7 @@
         <v>46238</v>
       </c>
       <c r="AA169" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB169" s="2" t="inlineStr">
         <is>
@@ -21590,7 +21600,7 @@
         <v>46238</v>
       </c>
       <c r="AA170" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB170" s="2" t="inlineStr">
         <is>
@@ -22368,7 +22378,7 @@
         <v>46254</v>
       </c>
       <c r="AA176" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB176" s="2" t="inlineStr">
         <is>
@@ -27704,7 +27714,7 @@
         <v>46229</v>
       </c>
       <c r="AA218" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB218" s="2" t="inlineStr">
         <is>
@@ -28732,7 +28742,7 @@
         <v>46254</v>
       </c>
       <c r="AA226" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB226" s="2" t="inlineStr">
         <is>
@@ -28866,7 +28876,7 @@
         <v>46258</v>
       </c>
       <c r="AA227" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB227" s="2" t="inlineStr">
         <is>
@@ -29008,7 +29018,7 @@
         <v>46254</v>
       </c>
       <c r="AA228" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB228" s="2" t="inlineStr">
         <is>
@@ -30210,7 +30220,7 @@
         <v>46258</v>
       </c>
       <c r="AA237" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB237" s="2" t="inlineStr">
         <is>
@@ -31589,7 +31599,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -31731,7 +31741,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -31966,7 +31976,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我局于2025年6月16日起,对你2020年1月1日-2020年12月31日期间的涉税情况进行检查,确认你有如下违法事实,并作出如下处罚决定: 根据《税务处理决定书》(鄂税三稽处〔2026〕8号)认定你存在以下违法事实: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 根据《中华人民共和国税收征收管理法》(2015年4月24日发布的主席令第二十三号修订)第六十四条第二款:“纳税人不进行纳税申报,不缴或者少缴应纳税款的,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 根据《内蒙古自治区国家税务局内蒙古自治区地方税务局关于发布〈内蒙古自治区税务行政处罚裁量基准〉的公告》(内蒙古自治区国家税务局内蒙古自治区地方税务局公告2017年第8号):“三、违反纳税申报管理类(三)纳税人不进行纳税申报,不缴或者少缴应纳税款的。 《中华人民共和国税收征收管理法》第六十四条第二款,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 1.不缴或者少缴税款100万元以下的,处百分之五十以上一倍以下罚款; ”之规定,决定对你个人不进行纳税申报造成少缴税款2,129.45元处以0.5倍罚款,即1,064.73元。</t>
+          <t>我局于2025年6月16日起,对你(地址:内蒙古鄂尔多斯市伊金霍洛旗纳林陶亥镇道劳岱村沟门社034号)2020年1月1日-2020年12月31日期间的涉税情况进行检查,违法事实及处理决定如下: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 ”之规定,对你少缴的个人所得税税款,按日加收滞纳税款万分之五的滞纳金。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -31974,13 +31984,15 @@
           <t>个人所得税</t>
         </is>
       </c>
-      <c r="R5" s="3" t="n"/>
+      <c r="R5" s="3" t="n">
+        <v>2129.45</v>
+      </c>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="n"/>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>综上所述,对你共处罚款1,064.73元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
+          <t>你在2020年应税收入为163,804.00元,应纳税额=163,804.00*1.3%=2,129.45元,应补缴个人所得税2,129.45元。 综上,你在2020年应税收入为163,804.00元,应补缴个人所得税2,129.45元,并就上述税款按日加收万分之五的滞纳金。</t>
         </is>
       </c>
       <c r="W5" s="4" t="n">
@@ -31994,7 +32006,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32037,7 +32049,7 @@
         <is>
           <t>Excel 与 CSV 历史数据已合并核对。 字段“官方原文链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/t20261013_898073.html”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202610/t20261013_898073.html”未静默覆盖。 字段“附件链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013417006903908.docx”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/tzgghhht/202610/P020261013417006903908.docx”未静默覆盖。 字段“页面标题”存在冲突:保留原值“国家税务总局内蒙古自治区税务局-
 旗县局通知公告”,新值“国家税务总局内蒙古自治区税务局-
-通知公告”未静默覆盖。</t>
+通知公告”未静默覆盖。 字段“主要违法事实”已根据官方附件重新解析。 字段“处理或处罚结果”已根据官方附件重新解析。 字段“附件链接”存在冲突:保留原值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013417006903908.docx”,新值“https://neimenggu.chinatax.gov.cn/sjpd/eeds/xjtzgghhht/202610/P020261013557090721134.docx”未静默覆盖。</t>
         </is>
       </c>
     </row>
@@ -32135,7 +32147,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -36348,7 +36360,7 @@
         <v>46234</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -39726,7 +39738,7 @@
         <v>46258</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -39868,7 +39880,7 @@
         <v>46254</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -40692,7 +40704,7 @@
         <v>46258</v>
       </c>
       <c r="AA70" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB70" s="2" t="inlineStr">
         <is>
@@ -41811,7 +41823,7 @@
         <v>46311</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -41851,7 +41863,7 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。</t>
+          <t>官方附件可下载,但尚未提取到可核实的案情或金额,按文号线索收录。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -41933,7 +41945,7 @@
         <v>46311</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -42055,7 +42067,7 @@
         <v>46311</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -42181,7 +42193,7 @@
         <v>46311</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -42215,7 +42227,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ5" s="2" t="inlineStr"/>
+      <c r="AJ5" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -42299,7 +42315,7 @@
         <v>46311</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -42333,7 +42349,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ6" s="2" t="inlineStr"/>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -42783,7 +42803,7 @@
         <v>46304</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -43145,7 +43165,7 @@
         <v>46308</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -45537,7 +45557,7 @@
         <v>46294</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -46155,7 +46175,7 @@
         <v>46296</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -46277,7 +46297,7 @@
         <v>46296</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -47119,7 +47139,7 @@
         <v>46286</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47241,7 +47261,7 @@
         <v>46286</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -47855,7 +47875,7 @@
         <v>46280</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -48087,7 +48107,7 @@
         <v>46280</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -48205,7 +48225,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -48319,7 +48339,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -48437,7 +48457,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -48555,7 +48575,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -52947,7 +52967,7 @@
         <v>46254</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -53073,7 +53093,7 @@
         <v>46254</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -55755,7 +55775,7 @@
         <v>46246</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -57601,7 +57621,7 @@
         <v>46238</v>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB132" s="2" t="inlineStr">
         <is>
@@ -57727,7 +57747,7 @@
         <v>46238</v>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB133" s="2" t="inlineStr">
         <is>
@@ -58083,7 +58103,7 @@
         <v>46254</v>
       </c>
       <c r="AA136" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB136" s="2" t="inlineStr">
         <is>
@@ -61003,7 +61023,7 @@
         <v>46229</v>
       </c>
       <c r="AA160" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
@@ -61625,7 +61645,7 @@
         <v>46254</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -62886,7 +62906,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -63012,7 +63032,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -63130,7 +63150,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -64163,7 +64183,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -64289,7 +64309,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -64407,7 +64427,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -64486,7 +64506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M194"/>
+  <dimension ref="A1:M195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -74196,8 +74216,57 @@
         </is>
       </c>
     </row>
+    <row r="195" ht="54" customHeight="1">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17T16:30:27+08:00</t>
+        </is>
+      </c>
+      <c r="B195" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10 至 2026-10-17</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="n">
+        <v>526</v>
+      </c>
+      <c r="D195" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E195" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G195" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H195" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I195" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L195" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='...</t>
+        </is>
+      </c>
+      <c r="M195" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问74页，访问失败437页，持久化待复核428个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M194"/>
+  <autoFilter ref="A1:M195"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-18
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$168</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -781,7 +781,7 @@
         <v>46311</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -903,7 +903,7 @@
         <v>46311</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
         <v>46311</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         <v>46311</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         <v>46311</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         <v>46308</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -1549,7 +1549,7 @@
         <v>46308</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -1814,7 +1814,7 @@
         <v>46308</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         <v>46308</v>
       </c>
       <c r="AA11" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
         <v>46304</v>
       </c>
       <c r="AA15" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
@@ -2812,7 +2812,7 @@
         <v>46308</v>
       </c>
       <c r="AA18" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
@@ -2978,7 +2978,7 @@
       </c>
       <c r="AJ19" s="2" t="inlineStr">
         <is>
-          <t>处理文书中的处罚结果串值已根据官方附件清除。</t>
+          <t>处理文书中的处罚结果串值已根据官方附件清除。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ20" s="2" t="inlineStr"/>
+      <c r="AJ20" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -6126,7 +6130,7 @@
         <v>46294</v>
       </c>
       <c r="AA45" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB45" s="2" t="inlineStr">
         <is>
@@ -6744,7 +6748,7 @@
         <v>46296</v>
       </c>
       <c r="AA50" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
@@ -6866,7 +6870,7 @@
         <v>46296</v>
       </c>
       <c r="AA51" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
@@ -8356,7 +8360,7 @@
         <v>46286</v>
       </c>
       <c r="AA63" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB63" s="2" t="inlineStr">
         <is>
@@ -8478,7 +8482,7 @@
         <v>46286</v>
       </c>
       <c r="AA64" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB64" s="2" t="inlineStr">
         <is>
@@ -9498,7 +9502,7 @@
         <v>46280</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -9730,7 +9734,7 @@
         <v>46280</v>
       </c>
       <c r="AA74" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB74" s="2" t="inlineStr">
         <is>
@@ -9848,7 +9852,7 @@
         <v>46280</v>
       </c>
       <c r="AA75" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB75" s="2" t="inlineStr">
         <is>
@@ -9962,7 +9966,7 @@
         <v>46280</v>
       </c>
       <c r="AA76" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB76" s="2" t="inlineStr">
         <is>
@@ -10080,7 +10084,7 @@
         <v>46280</v>
       </c>
       <c r="AA77" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB77" s="2" t="inlineStr">
         <is>
@@ -10198,7 +10202,7 @@
         <v>46280</v>
       </c>
       <c r="AA78" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB78" s="2" t="inlineStr">
         <is>
@@ -15210,7 +15214,7 @@
         <v>46254</v>
       </c>
       <c r="AA119" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB119" s="2" t="inlineStr">
         <is>
@@ -15336,7 +15340,7 @@
         <v>46254</v>
       </c>
       <c r="AA120" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB120" s="2" t="inlineStr">
         <is>
@@ -18276,7 +18280,7 @@
         <v>46246</v>
       </c>
       <c r="AA144" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB144" s="2" t="inlineStr">
         <is>
@@ -21614,7 +21618,7 @@
         <v>46234</v>
       </c>
       <c r="AA170" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB170" s="2" t="inlineStr">
         <is>
@@ -21736,7 +21740,7 @@
         <v>46238</v>
       </c>
       <c r="AA171" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB171" s="2" t="inlineStr">
         <is>
@@ -21862,7 +21866,7 @@
         <v>46238</v>
       </c>
       <c r="AA172" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB172" s="2" t="inlineStr">
         <is>
@@ -22640,7 +22644,7 @@
         <v>46254</v>
       </c>
       <c r="AA178" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB178" s="2" t="inlineStr">
         <is>
@@ -27976,7 +27980,7 @@
         <v>46229</v>
       </c>
       <c r="AA220" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB220" s="2" t="inlineStr">
         <is>
@@ -29004,7 +29008,7 @@
         <v>46254</v>
       </c>
       <c r="AA228" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB228" s="2" t="inlineStr">
         <is>
@@ -29138,7 +29142,7 @@
         <v>46258</v>
       </c>
       <c r="AA229" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB229" s="2" t="inlineStr">
         <is>
@@ -29280,7 +29284,7 @@
         <v>46254</v>
       </c>
       <c r="AA230" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB230" s="2" t="inlineStr">
         <is>
@@ -30482,7 +30486,7 @@
         <v>46258</v>
       </c>
       <c r="AA239" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB239" s="2" t="inlineStr">
         <is>
@@ -31863,7 +31867,7 @@
         <v>46308</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -32005,7 +32009,7 @@
         <v>46308</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -32270,7 +32274,7 @@
         <v>46308</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -32411,7 +32415,7 @@
         <v>46308</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -32584,7 +32588,7 @@
       </c>
       <c r="AJ7" s="2" t="inlineStr">
         <is>
-          <t>处理文书中的处罚结果串值已根据官方附件清除。</t>
+          <t>处理文书中的处罚结果串值已根据官方附件清除。 Excel 与 CSV 历史数据已合并核对。</t>
         </is>
       </c>
     </row>
@@ -32718,7 +32722,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -36886,7 +36894,7 @@
         <v>46234</v>
       </c>
       <c r="AA40" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
@@ -40264,7 +40272,7 @@
         <v>46258</v>
       </c>
       <c r="AA65" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB65" s="2" t="inlineStr">
         <is>
@@ -40406,7 +40414,7 @@
         <v>46254</v>
       </c>
       <c r="AA66" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB66" s="2" t="inlineStr">
         <is>
@@ -41230,7 +41238,7 @@
         <v>46258</v>
       </c>
       <c r="AA72" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB72" s="2" t="inlineStr">
         <is>
@@ -42351,7 +42359,7 @@
         <v>46311</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -42473,7 +42481,7 @@
         <v>46311</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -42595,7 +42603,7 @@
         <v>46311</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -42721,7 +42729,7 @@
         <v>46311</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -42843,7 +42851,7 @@
         <v>46311</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -43331,7 +43339,7 @@
         <v>46304</v>
       </c>
       <c r="AA10" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
@@ -43693,7 +43701,7 @@
         <v>46308</v>
       </c>
       <c r="AA13" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
@@ -46085,7 +46093,7 @@
         <v>46294</v>
       </c>
       <c r="AA33" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
@@ -46703,7 +46711,7 @@
         <v>46296</v>
       </c>
       <c r="AA38" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
@@ -46825,7 +46833,7 @@
         <v>46296</v>
       </c>
       <c r="AA39" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB39" s="2" t="inlineStr">
         <is>
@@ -47667,7 +47675,7 @@
         <v>46286</v>
       </c>
       <c r="AA46" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
@@ -47789,7 +47797,7 @@
         <v>46286</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
@@ -48403,7 +48411,7 @@
         <v>46280</v>
       </c>
       <c r="AA52" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB52" s="2" t="inlineStr">
         <is>
@@ -48635,7 +48643,7 @@
         <v>46280</v>
       </c>
       <c r="AA54" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
@@ -48753,7 +48761,7 @@
         <v>46280</v>
       </c>
       <c r="AA55" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB55" s="2" t="inlineStr">
         <is>
@@ -48867,7 +48875,7 @@
         <v>46280</v>
       </c>
       <c r="AA56" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB56" s="2" t="inlineStr">
         <is>
@@ -48985,7 +48993,7 @@
         <v>46280</v>
       </c>
       <c r="AA57" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB57" s="2" t="inlineStr">
         <is>
@@ -49103,7 +49111,7 @@
         <v>46280</v>
       </c>
       <c r="AA58" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB58" s="2" t="inlineStr">
         <is>
@@ -53495,7 +53503,7 @@
         <v>46254</v>
       </c>
       <c r="AA94" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB94" s="2" t="inlineStr">
         <is>
@@ -53621,7 +53629,7 @@
         <v>46254</v>
       </c>
       <c r="AA95" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB95" s="2" t="inlineStr">
         <is>
@@ -56303,7 +56311,7 @@
         <v>46246</v>
       </c>
       <c r="AA117" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB117" s="2" t="inlineStr">
         <is>
@@ -58149,7 +58157,7 @@
         <v>46238</v>
       </c>
       <c r="AA132" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB132" s="2" t="inlineStr">
         <is>
@@ -58275,7 +58283,7 @@
         <v>46238</v>
       </c>
       <c r="AA133" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB133" s="2" t="inlineStr">
         <is>
@@ -58631,7 +58639,7 @@
         <v>46254</v>
       </c>
       <c r="AA136" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB136" s="2" t="inlineStr">
         <is>
@@ -61551,7 +61559,7 @@
         <v>46229</v>
       </c>
       <c r="AA160" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB160" s="2" t="inlineStr">
         <is>
@@ -62173,7 +62181,7 @@
         <v>46254</v>
       </c>
       <c r="AA165" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB165" s="2" t="inlineStr">
         <is>
@@ -63434,7 +63442,7 @@
         <v>46238</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -63560,7 +63568,7 @@
         <v>46238</v>
       </c>
       <c r="AA5" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
@@ -63678,7 +63686,7 @@
         <v>46229</v>
       </c>
       <c r="AA6" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
@@ -64711,7 +64719,7 @@
         <v>46238</v>
       </c>
       <c r="AA2" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
@@ -64837,7 +64845,7 @@
         <v>46238</v>
       </c>
       <c r="AA3" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
@@ -64955,7 +64963,7 @@
         <v>46229</v>
       </c>
       <c r="AA4" s="4" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
@@ -65034,7 +65042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M196"/>
+  <dimension ref="A1:M197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -74846,8 +74854,57 @@
         </is>
       </c>
     </row>
+    <row r="197" ht="54" customHeight="1">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18T16:48:15+08:00</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-11 至 2026-10-18</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="n">
+        <v>531</v>
+      </c>
+      <c r="D197" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E197" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F197" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G197" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H197" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I197" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J197" s="2" t="inlineStr"/>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L197" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: https://fujian.chinatax.gov.cn/pingtanswj/zfxxgkzl/zfxxgkml/qtgg/: ConnectionError: HTTPSConnectionPool(host='fujian.chinatax.gov.cn', port=443): Max retries exceeded with url: /pingtanswj/zfxxgkzl/zfxxgkml/qtgg/ (Caused by NewConnectionError("HTTPSConnection(host='fujian...</t>
+        </is>
+      </c>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问76页，访问失败439页，持久化待复核430个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M196"/>
+  <autoFilter ref="A1:M197"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
data: update tax decisions 2026-10-19
</commit_message>
<xml_diff>
--- a/data/全国税务处理及行政处罚决定书汇总.xlsx
+++ b/data/全国税务处理及行政处罚决定书汇总.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'公告送达及文号线索'!$A$1:$AJ$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'待核验记录'!$A$1:$AJ$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'失效链接'!$A$1:$AJ$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'每日运行日志'!$A$1:$M$200</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -1709,7 +1709,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ9" s="2" t="inlineStr"/>
+      <c r="AJ9" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1827,7 +1831,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ10" s="2" t="inlineStr"/>
+      <c r="AJ10" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2020,7 +2028,7 @@
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>我局于2025年6月16日起,对你(地址:内蒙古鄂尔多斯市伊金霍洛旗纳林陶亥镇道劳岱村沟门社034号)2020年1月1日-2020年12月31日期间的涉税情况进行检查,违法事实及处理决定如下: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 ”之规定,对你少缴的个人所得税税款,按日加收滞纳税款万分之五的滞纳金。</t>
+          <t>我局于2025年6月16日起,对你2020年1月1日-2020年12月31日期间的涉税情况进行检查,确认你有如下违法事实,并作出如下处罚决定: 根据《税务处理决定书》(鄂税三稽处〔2026〕8号)认定你存在以下违法事实: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 根据《中华人民共和国税收征收管理法》(2015年4月24日发布的主席令第二十三号修订)第六十四条第二款:“纳税人不进行纳税申报,不缴或者少缴应纳税款的,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 根据《内蒙古自治区国家税务局内蒙古自治区地方税务局关于发布〈内蒙古自治区税务行政处罚裁量基准〉的公告》(内蒙古自治区国家税务局内蒙古自治区地方税务局公告2017年第8号):“三、违反纳税申报管理类(三)纳税人不进行纳税申报,不缴或者少缴应纳税款的。 《中华人民共和国税收征收管理法》第六十四条第二款,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 1.不缴或者少缴税款100万元以下的,处百分之五十以上一倍以下罚款; ”之规定,决定对你个人不进行纳税申报造成少缴税款2,129.45元处以0.5倍罚款,即1,064.73元。</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -2036,7 +2044,7 @@
       <c r="U12" s="3" t="n"/>
       <c r="V12" s="2" t="inlineStr">
         <is>
-          <t>你在2020年应税收入为163,804.00元,应纳税额=163,804.00*1.3%=2,129.45元,应补缴个人所得税2,129.45元。 综上,你在2020年应税收入为163,804.00元,应补缴个人所得税2,129.45元,并就上述税款按日加收万分之五的滞纳金。</t>
+          <t>综上所述,对你共处罚款1,064.73元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W12" s="4" t="n">
@@ -3178,7 +3186,7 @@
         <v>46312</v>
       </c>
       <c r="AA21" s="4" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
@@ -3314,7 +3322,7 @@
         <v>46312</v>
       </c>
       <c r="AA22" s="4" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="AB22" s="2" t="inlineStr">
         <is>
@@ -32482,7 +32490,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>我局于2025年6月16日起,对你(地址:内蒙古鄂尔多斯市伊金霍洛旗纳林陶亥镇道劳岱村沟门社034号)2020年1月1日-2020年12月31日期间的涉税情况进行检查,违法事实及处理决定如下: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 ”之规定,对你少缴的个人所得税税款,按日加收滞纳税款万分之五的滞纳金。</t>
+          <t>我局于2025年6月16日起,对你2020年1月1日-2020年12月31日期间的涉税情况进行检查,确认你有如下违法事实,并作出如下处罚决定: 根据《税务处理决定书》(鄂税三稽处〔2026〕8号)认定你存在以下违法事实: 经查,你于2020年提供装修服务取得收入163,804.00元,未进行纳税申报。 根据《中华人民共和国税收征收管理法》(2015年4月24日发布的主席令第二十三号修订)第六十四条第二款:“纳税人不进行纳税申报,不缴或者少缴应纳税款的,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 根据《内蒙古自治区国家税务局内蒙古自治区地方税务局关于发布〈内蒙古自治区税务行政处罚裁量基准〉的公告》(内蒙古自治区国家税务局内蒙古自治区地方税务局公告2017年第8号):“三、违反纳税申报管理类(三)纳税人不进行纳税申报,不缴或者少缴应纳税款的。 《中华人民共和国税收征收管理法》第六十四条第二款,由税务机关追缴其不缴或者少缴的税款、滞纳金,并处不缴或者少缴的税款百分之五十以上五倍以下的罚款。 1.不缴或者少缴税款100万元以下的,处百分之五十以上一倍以下罚款; ”之规定,决定对你个人不进行纳税申报造成少缴税款2,129.45元处以0.5倍罚款,即1,064.73元。</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -32498,7 +32506,7 @@
       <c r="U5" s="3" t="n"/>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>你在2020年应税收入为163,804.00元,应纳税额=163,804.00*1.3%=2,129.45元,应补缴个人所得税2,129.45元。 综上,你在2020年应税收入为163,804.00元,应补缴个人所得税2,129.45元,并就上述税款按日加收万分之五的滞纳金。</t>
+          <t>综上所述,对你共处罚款1,064.73元。 到期不缴纳罚款,我局可依照《中华人民共和国行政处罚法》第七十二条第一款第(一)项规定,每日按罚款数额的百分之三加处罚款。</t>
         </is>
       </c>
       <c r="W5" s="4" t="n">
@@ -32790,7 +32798,7 @@
         <v>46312</v>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
@@ -32926,7 +32934,7 @@
         <v>46312</v>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="AB8" s="2" t="inlineStr">
         <is>
@@ -43245,7 +43253,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ7" s="2" t="inlineStr"/>
+      <c r="AJ7" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -43363,7 +43375,11 @@
           <t>正常</t>
         </is>
       </c>
-      <c r="AJ8" s="2" t="inlineStr"/>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
+          <t>Excel 与 CSV 历史数据已合并核对。</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -65518,7 +65534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M199"/>
+  <dimension ref="A1:M200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -75481,8 +75497,57 @@
         </is>
       </c>
     </row>
+    <row r="200" ht="54" customHeight="1">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19T18:20:29+08:00</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12 至 2026-10-19</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="n">
+        <v>509</v>
+      </c>
+      <c r="D200" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E200" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G200" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H200" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I200" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J200" s="2" t="inlineStr"/>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>成功</t>
+        </is>
+      </c>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t>discover_official_index: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/: HTTPError: 403 Client Error: Forbidden for url: http://qinghai.chinatax.gov.cn/hxz/sjtzgg/ | discover_official_index: https://fujian.chinatax.gov.cn/fzsswj/xxgk/gsgg/qtl/: ConnectionError: HTTPSConnectionPool(host='fujian.chinat...</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>本次已核验来源新增0份文书；检索覆盖不完整，不能据此认定其他日期没有新文书。本轮可访问60页，访问失败447页，持久化待复核438个链接。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M199"/>
+  <autoFilter ref="A1:M200"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>

</xml_diff>